<commit_message>
Corrige les exportations 2024 avec le détail par société (Tableau 26)
Le Tableau 25 utilisé initialement agrège les exportations 2024 par pays
sans indiquer la société. Le rapport complet contient un Tableau 26
("Détail des exportations désagrégé par substances") qui donne la société
et le projet pour chaque ligne, avec des totaux par substance identiques
à ceux du Tableau 25. Remplace les 46 lignes 2024 (dont plusieurs "NC" en
société) par les 50 lignes désagrégées du Tableau 26.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -9486,7 +9486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G780"/>
+  <dimension ref="A1:G784"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="6.7265625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -32287,28 +32287,28 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>ICS</t>
+          <t>PMC</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE</t>
+          <t>Or</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Onces</t>
         </is>
       </c>
       <c r="E735" t="n">
-        <v>470216</v>
+        <v>121623</v>
       </c>
       <c r="F735" t="n">
-        <v>279802568290</v>
+        <v>176892827875</v>
       </c>
       <c r="G735" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Australie</t>
         </is>
       </c>
     </row>
@@ -32318,28 +32318,28 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SGO</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Or</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>Onces</t>
         </is>
       </c>
       <c r="E736" t="n">
-        <v>94451</v>
+        <v>116418</v>
       </c>
       <c r="F736" t="n">
-        <v>7691623558</v>
+        <v>171988995312</v>
       </c>
       <c r="G736" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Dubai</t>
         </is>
       </c>
     </row>
@@ -32349,7 +32349,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SGO</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
@@ -32363,14 +32363,14 @@
         </is>
       </c>
       <c r="E737" t="n">
-        <v>116418</v>
+        <v>105001</v>
       </c>
       <c r="F737" t="n">
-        <v>171988995312</v>
+        <v>153070817850</v>
       </c>
       <c r="G737" t="inlineStr">
         <is>
-          <t>Émirats Arabes Unis (Dubai)</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -32385,7 +32385,7 @@
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
@@ -32394,14 +32394,14 @@
         </is>
       </c>
       <c r="E738" t="n">
-        <v>13177</v>
+        <v>470216</v>
       </c>
       <c r="F738" t="n">
-        <v>7716598633</v>
+        <v>279802568290</v>
       </c>
       <c r="G738" t="inlineStr">
         <is>
-          <t>Émirats Arabes Unis (Dubai)</t>
+          <t>INDE</t>
         </is>
       </c>
     </row>
@@ -32416,7 +32416,7 @@
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>PHOSPHATE MONO AMMONIQUE</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
@@ -32425,14 +32425,14 @@
         </is>
       </c>
       <c r="E739" t="n">
-        <v>13504</v>
+        <v>13177</v>
       </c>
       <c r="F739" t="n">
-        <v>5078254628</v>
+        <v>7716598633</v>
       </c>
       <c r="G739" t="inlineStr">
         <is>
-          <t>Émirats Arabes Unis (Dubai)</t>
+          <t>Dubai</t>
         </is>
       </c>
     </row>
@@ -32442,28 +32442,28 @@
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>CDS</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>Argent</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E740" t="n">
-        <v>8904</v>
+        <v>1196672</v>
       </c>
       <c r="F740" t="n">
-        <v>156146734</v>
+        <v>56914606200</v>
       </c>
       <c r="G740" t="inlineStr">
         <is>
-          <t>Émirats Arabes Unis (Dubai)</t>
+          <t>zone uemoa</t>
         </is>
       </c>
     </row>
@@ -32473,28 +32473,28 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>CDS</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>Or</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E741" t="n">
-        <v>121623</v>
+        <v>320386</v>
       </c>
       <c r="F741" t="n">
-        <v>176892827875</v>
+        <v>15314992585</v>
       </c>
       <c r="G741" t="inlineStr">
         <is>
-          <t>Australie</t>
+          <t>zone hors uemoa</t>
         </is>
       </c>
     </row>
@@ -32504,28 +32504,28 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>Argent</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E742" t="n">
-        <v>10095</v>
+        <v>99563</v>
       </c>
       <c r="F742" t="n">
-        <v>169980320</v>
+        <v>10819242900</v>
       </c>
       <c r="G742" t="inlineStr">
         <is>
-          <t>Australie</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32535,12 +32535,12 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
@@ -32549,14 +32549,14 @@
         </is>
       </c>
       <c r="E743" t="n">
-        <v>387783</v>
+        <v>102356</v>
       </c>
       <c r="F743" t="n">
-        <v>57119016447</v>
+        <v>5152601247</v>
       </c>
       <c r="G743" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32566,12 +32566,12 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
@@ -32580,14 +32580,14 @@
         </is>
       </c>
       <c r="E744" t="n">
-        <v>39376</v>
+        <v>21001</v>
       </c>
       <c r="F744" t="n">
-        <v>43681219368</v>
+        <v>1023768387</v>
       </c>
       <c r="G744" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Gambia</t>
         </is>
       </c>
     </row>
@@ -32597,12 +32597,12 @@
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
@@ -32611,14 +32611,14 @@
         </is>
       </c>
       <c r="E745" t="n">
-        <v>27523</v>
+        <v>16340</v>
       </c>
       <c r="F745" t="n">
-        <v>28804344792</v>
+        <v>498575000</v>
       </c>
       <c r="G745" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Gambia</t>
         </is>
       </c>
     </row>
@@ -32628,12 +32628,12 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D746" t="inlineStr">
@@ -32642,14 +32642,14 @@
         </is>
       </c>
       <c r="E746" t="n">
-        <v>153286</v>
+        <v>7013</v>
       </c>
       <c r="F746" t="n">
-        <v>26445296560</v>
+        <v>410459933</v>
       </c>
       <c r="G746" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Mauritanie</t>
         </is>
       </c>
     </row>
@@ -32659,12 +32659,12 @@
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
@@ -32673,14 +32673,14 @@
         </is>
       </c>
       <c r="E747" t="n">
-        <v>6092</v>
+        <v>25717</v>
       </c>
       <c r="F747" t="n">
-        <v>4539903428</v>
+        <v>227326200</v>
       </c>
       <c r="G747" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>GUINEE BISSAU</t>
         </is>
       </c>
     </row>
@@ -32690,12 +32690,12 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
@@ -32704,14 +32704,14 @@
         </is>
       </c>
       <c r="E748" t="n">
-        <v>31443</v>
+        <v>3989</v>
       </c>
       <c r="F748" t="n">
-        <v>4311499782</v>
+        <v>191512400</v>
       </c>
       <c r="G748" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Cap-Vert</t>
         </is>
       </c>
     </row>
@@ -32721,12 +32721,12 @@
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
@@ -32735,14 +32735,14 @@
         </is>
       </c>
       <c r="E749" t="n">
-        <v>2640</v>
+        <v>320</v>
       </c>
       <c r="F749" t="n">
-        <v>2861618508</v>
+        <v>15360000</v>
       </c>
       <c r="G749" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Guinée</t>
         </is>
       </c>
     </row>
@@ -32752,12 +32752,12 @@
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>GCO</t>
+          <t>SOMIVA</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>ILMENITE 56</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
@@ -32766,14 +32766,14 @@
         </is>
       </c>
       <c r="E750" t="n">
-        <v>20001</v>
+        <v>121573</v>
       </c>
       <c r="F750" t="n">
-        <v>2761143939</v>
+        <v>10898420355</v>
       </c>
       <c r="G750" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>Switzerland</t>
         </is>
       </c>
     </row>
@@ -32783,12 +32783,12 @@
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>SSPT</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>Attapulgite</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D751" t="inlineStr">
@@ -32797,14 +32797,14 @@
         </is>
       </c>
       <c r="E751" t="n">
-        <v>59499</v>
+        <v>94451</v>
       </c>
       <c r="F751" t="n">
-        <v>1642761360</v>
+        <v>7691623558</v>
       </c>
       <c r="G751" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>INDE</t>
         </is>
       </c>
     </row>
@@ -32814,28 +32814,28 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SOMIVA</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>Or</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D752" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E752" t="n">
-        <v>105001</v>
+        <v>72510</v>
       </c>
       <c r="F752" t="n">
-        <v>153070817850</v>
+        <v>6046547100</v>
       </c>
       <c r="G752" t="inlineStr">
         <is>
-          <t>Suisse</t>
+          <t>SWITZERLAND</t>
         </is>
       </c>
     </row>
@@ -32845,28 +32845,28 @@
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SOMIVA</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>Argent</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E753" t="n">
-        <v>8181</v>
+        <v>30152</v>
       </c>
       <c r="F753" t="n">
-        <v>140740539</v>
+        <v>2643705806</v>
       </c>
       <c r="G753" t="inlineStr">
         <is>
-          <t>Suisse</t>
+          <t>PAYS BAS</t>
         </is>
       </c>
     </row>
@@ -32876,12 +32876,12 @@
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
@@ -32890,14 +32890,14 @@
         </is>
       </c>
       <c r="E754" t="n">
-        <v>1196672</v>
+        <v>29612</v>
       </c>
       <c r="F754" t="n">
-        <v>56914606200</v>
+        <v>1885932032</v>
       </c>
       <c r="G754" t="inlineStr">
         <is>
-          <t>zone uemoa</t>
+          <t>INDONESIA</t>
         </is>
       </c>
     </row>
@@ -32907,12 +32907,12 @@
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D755" t="inlineStr">
@@ -32921,14 +32921,14 @@
         </is>
       </c>
       <c r="E755" t="n">
-        <v>201919</v>
+        <v>25084</v>
       </c>
       <c r="F755" t="n">
-        <v>15971844147</v>
+        <v>1493949967</v>
       </c>
       <c r="G755" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>BRAZIL</t>
         </is>
       </c>
     </row>
@@ -32938,28 +32938,28 @@
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>ICS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>NPK - Sac 50Kg</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D756" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E756" t="n">
-        <v>14658</v>
+        <v>21169</v>
       </c>
       <c r="F756" t="n">
-        <v>4644684890</v>
+        <v>1227500356</v>
       </c>
       <c r="G756" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -32969,28 +32969,28 @@
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>ICS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C757" t="inlineStr">
         <is>
-          <t>DAP - Sac 50Kg</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D757" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E757" t="n">
-        <v>1980</v>
+        <v>2925</v>
       </c>
       <c r="F757" t="n">
-        <v>792000000</v>
+        <v>358792082</v>
       </c>
       <c r="G757" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>GHANA</t>
         </is>
       </c>
     </row>
@@ -33000,7 +33000,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SOMIVA</t>
         </is>
       </c>
       <c r="C758" t="inlineStr">
@@ -33031,28 +33031,28 @@
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>ICS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C759" t="inlineStr">
         <is>
-          <t>DSP - Sac 50 Kg</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D759" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E759" t="n">
-        <v>1061</v>
+        <v>3888</v>
       </c>
       <c r="F759" t="n">
-        <v>90185000</v>
+        <v>150018417</v>
       </c>
       <c r="G759" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>Italie</t>
         </is>
       </c>
     </row>
@@ -33062,28 +33062,28 @@
       </c>
       <c r="B760" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>ICS</t>
         </is>
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>PHOSPHATE MONO AMMONIQUE</t>
         </is>
       </c>
       <c r="D760" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="E760" t="n">
-        <v>121573</v>
+        <v>32978</v>
       </c>
       <c r="F760" t="n">
-        <v>10898420355</v>
+        <v>14570824067</v>
       </c>
       <c r="G760" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>United States</t>
         </is>
       </c>
     </row>
@@ -33124,28 +33124,28 @@
       </c>
       <c r="B762" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>ICS</t>
         </is>
       </c>
       <c r="C762" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>PHOSPHATE MONO AMMONIQUE</t>
         </is>
       </c>
       <c r="D762" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="E762" t="n">
-        <v>320386</v>
+        <v>13504</v>
       </c>
       <c r="F762" t="n">
-        <v>15314992585</v>
+        <v>5078254628</v>
       </c>
       <c r="G762" t="inlineStr">
         <is>
-          <t>zone hors uemoa</t>
+          <t>Dubai</t>
         </is>
       </c>
     </row>
@@ -33155,28 +33155,28 @@
       </c>
       <c r="B763" t="inlineStr">
         <is>
-          <t>ICS</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>PHOSPHATE MONO AMMONIQUE</t>
+          <t>ILMENITE 54</t>
         </is>
       </c>
       <c r="D763" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E763" t="n">
-        <v>32978</v>
+        <v>387783</v>
       </c>
       <c r="F763" t="n">
-        <v>14570824067</v>
+        <v>57119016447</v>
       </c>
       <c r="G763" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33186,7 +33186,7 @@
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>BMCC</t>
         </is>
       </c>
       <c r="C764" t="inlineStr">
@@ -33217,28 +33217,28 @@
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>ICS</t>
         </is>
       </c>
       <c r="C765" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>NPK - Sac 50Kg</t>
         </is>
       </c>
       <c r="D765" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="E765" t="n">
-        <v>365862</v>
+        <v>14658</v>
       </c>
       <c r="F765" t="n">
-        <v>3493161900</v>
+        <v>4644684890</v>
       </c>
       <c r="G765" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -33279,12 +33279,12 @@
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SSPT</t>
         </is>
       </c>
       <c r="C767" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Attapuglite</t>
         </is>
       </c>
       <c r="D767" t="inlineStr">
@@ -33293,14 +33293,14 @@
         </is>
       </c>
       <c r="E767" t="n">
-        <v>37341</v>
+        <v>59499</v>
       </c>
       <c r="F767" t="n">
-        <v>1522343387</v>
+        <v>1642761360</v>
       </c>
       <c r="G767" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33310,12 +33310,12 @@
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SSPT</t>
         </is>
       </c>
       <c r="C768" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Attapuglite</t>
         </is>
       </c>
       <c r="D768" t="inlineStr">
@@ -33324,14 +33324,14 @@
         </is>
       </c>
       <c r="E768" t="n">
-        <v>72510</v>
+        <v>66541</v>
       </c>
       <c r="F768" t="n">
-        <v>6046547100</v>
+        <v>1622901908</v>
       </c>
       <c r="G768" t="inlineStr">
         <is>
-          <t>SWITZERLAND</t>
+          <t>United Kingdom</t>
         </is>
       </c>
     </row>
@@ -33341,12 +33341,12 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>SSPT</t>
         </is>
       </c>
       <c r="C769" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Attapuglite</t>
         </is>
       </c>
       <c r="D769" t="inlineStr">
@@ -33355,10 +33355,10 @@
         </is>
       </c>
       <c r="E769" t="n">
-        <v>30152</v>
+        <v>30502</v>
       </c>
       <c r="F769" t="n">
-        <v>2643705806</v>
+        <v>918624505</v>
       </c>
       <c r="G769" t="inlineStr">
         <is>
@@ -33372,12 +33372,12 @@
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>SSPT</t>
+          <t>GECAMINE</t>
         </is>
       </c>
       <c r="C770" t="inlineStr">
         <is>
-          <t>Attapulgite</t>
+          <t>BASALTE</t>
         </is>
       </c>
       <c r="D770" t="inlineStr">
@@ -33386,14 +33386,14 @@
         </is>
       </c>
       <c r="E770" t="n">
-        <v>30502</v>
+        <v>340661</v>
       </c>
       <c r="F770" t="n">
-        <v>918624505</v>
+        <v>3071169676</v>
       </c>
       <c r="G770" t="inlineStr">
         <is>
-          <t>PAYS BAS</t>
+          <t>Gambia</t>
         </is>
       </c>
     </row>
@@ -33403,28 +33403,30 @@
       </c>
       <c r="B771" t="inlineStr">
         <is>
+          <t>TALIX</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>BASALTE</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="C771" t="inlineStr">
-        <is>
-          <t>Phosphate de chaux naturel</t>
-        </is>
-      </c>
-      <c r="D771" t="inlineStr">
-        <is>
-          <t>Tonne</t>
-        </is>
-      </c>
-      <c r="E771" t="n">
-        <v>29612</v>
-      </c>
       <c r="F771" t="n">
-        <v>1885932032</v>
+        <v>358807621</v>
       </c>
       <c r="G771" t="inlineStr">
         <is>
-          <t>INDONESIA</t>
+          <t>Gambia</t>
         </is>
       </c>
     </row>
@@ -33434,12 +33436,12 @@
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>SSPT</t>
+          <t>COGECA</t>
         </is>
       </c>
       <c r="C772" t="inlineStr">
         <is>
-          <t>Attapulgite</t>
+          <t>BASALTE</t>
         </is>
       </c>
       <c r="D772" t="inlineStr">
@@ -33448,14 +33450,14 @@
         </is>
       </c>
       <c r="E772" t="n">
-        <v>66541</v>
+        <v>25201</v>
       </c>
       <c r="F772" t="n">
-        <v>1622901908</v>
+        <v>63184603</v>
       </c>
       <c r="G772" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Gambia</t>
         </is>
       </c>
     </row>
@@ -33465,12 +33467,12 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C773" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>ZIRCON MEDIUM</t>
         </is>
       </c>
       <c r="D773" t="inlineStr">
@@ -33479,14 +33481,14 @@
         </is>
       </c>
       <c r="E773" t="n">
-        <v>25084</v>
+        <v>31443</v>
       </c>
       <c r="F773" t="n">
-        <v>1493949967</v>
+        <v>4311499782</v>
       </c>
       <c r="G773" t="inlineStr">
         <is>
-          <t>BRAZIL</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33496,12 +33498,12 @@
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>LEUCOXENE</t>
         </is>
       </c>
       <c r="D774" t="inlineStr">
@@ -33510,14 +33512,14 @@
         </is>
       </c>
       <c r="E774" t="n">
-        <v>21169</v>
+        <v>6092</v>
       </c>
       <c r="F774" t="n">
-        <v>1227500356</v>
+        <v>4539903428</v>
       </c>
       <c r="G774" t="inlineStr">
         <is>
-          <t>Espagne</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33527,12 +33529,12 @@
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>RUTILE</t>
         </is>
       </c>
       <c r="D775" t="inlineStr">
@@ -33541,14 +33543,14 @@
         </is>
       </c>
       <c r="E775" t="n">
-        <v>7013</v>
+        <v>2640</v>
       </c>
       <c r="F775" t="n">
-        <v>410459933</v>
+        <v>2861618508</v>
       </c>
       <c r="G775" t="inlineStr">
         <is>
-          <t>Mauritanie</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33558,12 +33560,12 @@
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>ILMENITE 56</t>
         </is>
       </c>
       <c r="D776" t="inlineStr">
@@ -33572,14 +33574,14 @@
         </is>
       </c>
       <c r="E776" t="n">
-        <v>2925</v>
+        <v>20001</v>
       </c>
       <c r="F776" t="n">
-        <v>358792082</v>
+        <v>2761143939</v>
       </c>
       <c r="G776" t="inlineStr">
         <is>
-          <t>GHANA</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33589,12 +33591,12 @@
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>ZIRCON PREMIUM</t>
         </is>
       </c>
       <c r="D777" t="inlineStr">
@@ -33603,14 +33605,14 @@
         </is>
       </c>
       <c r="E777" t="n">
-        <v>25717</v>
+        <v>39376</v>
       </c>
       <c r="F777" t="n">
-        <v>227326200</v>
+        <v>43681219368</v>
       </c>
       <c r="G777" t="inlineStr">
         <is>
-          <t>GUINEE BISSAU</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33620,12 +33622,12 @@
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>ZIRCON STANDARD</t>
         </is>
       </c>
       <c r="D778" t="inlineStr">
@@ -33634,14 +33636,14 @@
         </is>
       </c>
       <c r="E778" t="n">
-        <v>3989</v>
+        <v>27523</v>
       </c>
       <c r="F778" t="n">
-        <v>191512400</v>
+        <v>28804344792</v>
       </c>
       <c r="G778" t="inlineStr">
         <is>
-          <t>Cap-Vert</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33651,12 +33653,12 @@
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>GCO</t>
         </is>
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>ILMENITE 58</t>
         </is>
       </c>
       <c r="D779" t="inlineStr">
@@ -33665,14 +33667,14 @@
         </is>
       </c>
       <c r="E779" t="n">
-        <v>3888</v>
+        <v>153286</v>
       </c>
       <c r="F779" t="n">
-        <v>150018417</v>
+        <v>26445296560</v>
       </c>
       <c r="G779" t="inlineStr">
         <is>
-          <t>Italie</t>
+          <t>FRANCE</t>
         </is>
       </c>
     </row>
@@ -33682,28 +33684,152 @@
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>ICS</t>
         </is>
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>DAP - Sac 50Kg</t>
         </is>
       </c>
       <c r="D780" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="E780" t="n">
-        <v>320</v>
+        <v>1980</v>
       </c>
       <c r="F780" t="n">
-        <v>15360000</v>
+        <v>792000000</v>
       </c>
       <c r="G780" t="inlineStr">
         <is>
-          <t>Guinée</t>
+          <t>Mali</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>PMC</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Argent</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Onces</t>
+        </is>
+      </c>
+      <c r="E781" t="n">
+        <v>10095</v>
+      </c>
+      <c r="F781" t="n">
+        <v>169980320</v>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>Australie</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>SGO</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Argent</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Onces</t>
+        </is>
+      </c>
+      <c r="E782" t="n">
+        <v>8904</v>
+      </c>
+      <c r="F782" t="n">
+        <v>156146734</v>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>SGO</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Argent</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Onces</t>
+        </is>
+      </c>
+      <c r="E783" t="n">
+        <v>8181</v>
+      </c>
+      <c r="F783" t="n">
+        <v>140740539</v>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>Suisse</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>DSP - Sac 50 Kg</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="E784" t="n">
+        <v>1061</v>
+      </c>
+      <c r="F784" t="n">
+        <v>90185000</v>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>Mali</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajoute une feuille Notes méthodologiques
Documente la portée (secteur minier uniquement), les sources par année,
les conventions de codage (NC, N/A, USD) et la limite connue sur les
exportations 2021 (page manquante dans l'extrait PDF source), avec le
lien vers le rapport complet pour compléter cette année ultérieurement.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -6,8 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="production" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="exportation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="production" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="exportation" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +60,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,6 +448,200 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Notes méthodologiques - Données sur la production et les ventes (secteur minier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Portée</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Les feuilles "production" et "exportation" couvrent uniquement le secteur MINIER du Sénégal, de 2014 à 2024. Le secteur des hydrocarbures (pétrole, gaz, PETROSEN) n'est pas inclus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sources par année</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2014 à 2018</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Annexe 9 "Données sur la production et les ventes/exportations" des rapports ITIE Sénégal annuels (tableau unique combinant production et exportation par société).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2019 à 2021</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tableaux "Détail des productions du secteur minier" et "Détail des exportations et ventes locales du secteur minier" des rapports ITIE Sénégal 2019-2021 (numérotation Tableau 32/33 selon les années).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Tableaux 46 (production) et 47 (exportations) du rapport ITIE Sénégal 2022.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tableaux 18 (production) et 19 (exportations) du rapport ITIE Sénégal 2023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Tableau 22 (production) et Tableau 26 (exportations désagrégées par société et projet) du rapport ITIE Sénégal 2024. Le Tableau 25, plus visible mais agrégé par pays uniquement, n'a pas été utilisé pour l'exportation car il ne mentionne pas la société ; ses totaux par substance concordent avec ceux du Tableau 26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Conventions et codes utilisés</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Donnée non communiquée par la société ou l'administration (telle qu'indiquée dans le rapport source : "NC", "n/c", "N/C").</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sous-produit non destiné à la vente (utilisé comme intrant, par ex. pour la production de ciment), tel qu'indiqué dans le rapport source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Valeurs suivies de "USD"</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Certaines valeurs de production (notamment GCO 2014-2016) sont exprimées en dollars US dans le rapport source plutôt qu'en FCFA ; elles ont été conservées telles quelles avec la mention "USD" plutôt que d'être converties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Nombres avec virgule (ex. 12,5)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Décimales telles que rapportées à la source (les rapports 2020-2021 expriment certaines valeurs de production en milliards de FCFA arrondis, converties ici en FCFA entiers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Limite connue : exportations 2021 incomplètes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Le fichier source 2021.pdf fourni est un extrait de 5 pages du rapport ITIE 2021 complet. Le tableau des exportations (Tableau 33) y est tronqué : il s'arrête après la ligne "Leucoxène / GCO / Dubaï" et il manque la suite (Rutile, Zircon Premium, Zircon Standard, Medium Grade Zircon Sand, Sables minéralisés et autres substances), ainsi que les totaux par substance et le total général. Seules les lignes visibles dans l'extrait disponible ont été intégrées dans la feuille "exportation" pour l'année 2021.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pour compléter cette année, il faut le rapport ITIE Sénégal 2021 complet (ou la page manquante du Tableau 33) : https://donnees.itie.sn/wp-content/uploads/2022/12/Rapport-ITIE-Senegal-2021-Final-21-12-2022-Signe.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F338"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
@@ -9480,7 +9697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Harmonise les noms de sociétés et de types de minerai
Unifie les variantes de casse/orthographe (SOCOCIM/SOCOCIM INDUSTRIES,
DANGOTE/Dangote, GECAMINES/GECAMINE/Gécamines, Ilmenite 54/ILMENITE 54/
Ilménite 54%, Zircon Premium/Premium Zircon, Attapulgite/Attapulgide, etc.)
en un seul libellé canonique par société et par minerai sur les deux
feuilles, sans fusionner les grades/produits réellement distincts
(Phosphate Naturel, Phosphate de chaux naturel, Phosphate tricalcique...).
Documente la convention dans la feuille Notes.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -62,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -75,6 +75,7 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -643,6 +644,20 @@
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Le fichier source 2021.pdf initialement fourni (extrait de 5 pages) était tronqué : il manquait une page du Tableau 33 (fin du Leucoxène, Zircon Standard, Medium Grade Zircon, Zircon Premium, Rutile, et la catégorie "Autre"/SOCOCIM). Cette page manquante a été fournie séparément et intégrée à la feuille exportation. Les lignes de totaux par substance et le total général du tableau source n'ont pas été reportés (seules les lignes détaillées par opérateur/pays figurent dans la feuille).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Harmonisation des noms de sociétés et de types de minerai</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel, ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%"). Ces variantes ont été harmonisées en un seul libellé par société et par minerai, pour permettre des tableaux croisés dynamiques fiables. Les libellés décrivant des grades ou produits réellement différents (ex : "Phosphate", "Phosphate Naturel", "Phosphate de chaux naturel", "Phosphate tricalcique", "Phosphate Sec Criblé") ont été conservés distincts, de même que les agrégats spécifiques à certaines années ("Minerais de titane", "Titane", "Sables minéralisés").</t>
         </is>
       </c>
     </row>
@@ -716,7 +731,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>marno-calcaire</t>
+          <t>Marno-Calcaire</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -749,7 +764,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>calcaire</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -978,7 +993,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1009,7 +1024,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1040,7 +1055,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1071,7 +1086,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1133,7 +1148,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1352,7 +1367,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Phosphate sec criblé</t>
+          <t>Phosphate Sec Criblé</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1383,7 +1398,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1634,7 +1649,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1835,7 +1850,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1866,7 +1881,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1897,7 +1912,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1928,7 +1943,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1990,7 +2005,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2178,7 +2193,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Laterite</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2493,7 +2508,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2694,7 +2709,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2725,7 +2740,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2756,7 +2771,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2787,7 +2802,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2880,7 +2895,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3068,7 +3083,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Laterite</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3387,7 +3402,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3418,7 +3433,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3648,7 +3663,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3679,7 +3694,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3710,7 +3725,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3741,7 +3756,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3772,7 +3787,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3803,7 +3818,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3834,7 +3849,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3958,7 +3973,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>calcaire</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3989,7 +4004,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>argile</t>
+          <t>Argile</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -4020,7 +4035,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>latérite</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -4272,7 +4287,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>marno-calcaire</t>
+          <t>Marno-Calcaire</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4303,7 +4318,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>calcaire</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4623,7 +4638,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ATTAPULGITE</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4654,7 +4669,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -4687,7 +4702,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE ET ACIDES POLYPHOSPHORIQUES</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -4722,7 +4737,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -4757,7 +4772,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Phosphate diammonique</t>
+          <t>DAP (Phosphate Diammonique)</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -4787,12 +4802,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>calcaire</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -4818,12 +4833,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>argile</t>
+          <t>Argile</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -4849,12 +4864,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>latérite</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -4880,7 +4895,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4915,7 +4930,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -4986,7 +5001,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -5079,7 +5094,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -5110,7 +5125,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -5451,7 +5466,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -5482,7 +5497,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sands</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -5544,7 +5559,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Zircon premium</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -5575,7 +5590,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Zircon standard</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -5601,7 +5616,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -5632,7 +5647,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -5663,7 +5678,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -5694,7 +5709,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Gécamines</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -5761,7 +5776,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Engrais chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -5885,7 +5900,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Phosphate de chaux</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -6195,7 +6210,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Ilménite 54%</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -6226,7 +6241,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ilménite 56%</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -6257,7 +6272,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -6350,7 +6365,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -6536,7 +6551,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Attapulgites</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -6660,7 +6675,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Marnes</t>
+          <t>Marne</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -6691,7 +6706,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Latérites</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -6753,7 +6768,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Latérites</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -7042,7 +7057,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Ilménite 54%</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -7073,7 +7088,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Ilménite 56%</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -7104,7 +7119,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -7197,7 +7212,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -7290,7 +7305,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Phosphate de chaux</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -7321,7 +7336,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Acide phosphorique</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -7352,7 +7367,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Phosphate de chaux</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -7383,7 +7398,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Phosphate de chaux</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -7973,7 +7988,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -8035,7 +8050,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -8071,7 +8086,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -8285,7 +8300,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Gécamines</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -8352,7 +8367,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -8440,7 +8455,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Gécamines</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -8540,7 +8555,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Ilmenite 56</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -8571,7 +8586,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Zircon Sand Medium</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -8597,12 +8612,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Sephos/G-PHOS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Phosphate Sec Crible</t>
+          <t>Phosphate Sec Criblé</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -8633,7 +8648,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -8788,7 +8803,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Laterite</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -8819,7 +8834,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Laterite</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -8885,7 +8900,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Manganese</t>
+          <t>Manganèse</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -8980,7 +8995,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -9011,7 +9026,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>CLINKER</t>
+          <t>Clinker</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -9042,7 +9057,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>MARNO-CALCAIRE</t>
+          <t>Marno-Calcaire</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -9075,7 +9090,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -9108,7 +9123,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -9141,7 +9156,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>LATERITE</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -9236,7 +9251,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -9267,7 +9282,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -9298,7 +9313,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -9329,7 +9344,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -9360,7 +9375,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -9391,7 +9406,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -9422,7 +9437,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -9453,7 +9468,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>ILMENITE 56</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -9484,7 +9499,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -9515,7 +9530,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>CLINKER</t>
+          <t>Clinker</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -9577,7 +9592,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>PHOSPHATE NATUREL</t>
+          <t>Phosphate Naturel</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -9608,7 +9623,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>PHOSPHATE SEC CRIBLE</t>
+          <t>Phosphate Sec Criblé</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -9639,7 +9654,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>ATTAPULGITE</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -9670,7 +9685,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>ATTAPULGITE</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -9701,7 +9716,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -9732,7 +9747,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -9765,7 +9780,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -9798,7 +9813,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ARGILE</t>
+          <t>Argile</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -9831,7 +9846,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>LATERITE</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -9864,7 +9879,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -9897,7 +9912,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -9925,12 +9940,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>GECAMINE</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -9958,12 +9973,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>GECAMINE</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -9996,7 +10011,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -10029,7 +10044,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>MINERAUX LOURDS</t>
+          <t>Minéraux lourds</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -10062,7 +10077,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>HORMITE</t>
+          <t>Hormite</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -10095,7 +10110,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>ATTAPULGITE</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -10128,7 +10143,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>Or</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -10161,7 +10176,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>ARGENT</t>
+          <t>Argent</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -10194,7 +10209,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -10225,7 +10240,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -10256,7 +10271,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>ENGRAIS</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -10349,7 +10364,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
@@ -10380,7 +10395,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>CLINKER</t>
+          <t>Clinker</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -10411,7 +10426,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>MARNO-CALCAIRE</t>
+          <t>Marno-Calcaire</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -10442,7 +10457,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -10473,7 +10488,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -10504,7 +10519,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>LATERITE</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -10535,7 +10550,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>CIMENT</t>
+          <t>Ciment</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -10566,7 +10581,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>CLINKER</t>
+          <t>Clinker</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -10597,7 +10612,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -10628,7 +10643,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -10659,7 +10674,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -10690,7 +10705,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -10721,7 +10736,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -10752,7 +10767,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -10783,7 +10798,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -10814,7 +10829,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>ILMENITE 56</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -10876,7 +10891,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>PHOSPHATE NATUREL</t>
+          <t>Phosphate Naturel</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -10907,7 +10922,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>PHOSPHATE SEC CRIBLE</t>
+          <t>Phosphate Sec Criblé</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -10969,7 +10984,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Phosphates</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -11000,7 +11015,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -11033,7 +11048,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -11066,7 +11081,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>ARGILE</t>
+          <t>Argile</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -11099,7 +11114,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>LATERITE</t>
+          <t>Latérite</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -11132,7 +11147,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -11165,7 +11180,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -11193,12 +11208,12 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>GECAMINE</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -11226,12 +11241,12 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>GECAMINE</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>CALCAIRE</t>
+          <t>Calcaire</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -11264,7 +11279,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -11297,7 +11312,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>OR + Argent</t>
+          <t>Or + Argent</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -11888,7 +11903,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -11919,7 +11934,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -11950,7 +11965,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -11981,7 +11996,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -12012,7 +12027,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -12043,7 +12058,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -12074,7 +12089,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -12105,7 +12120,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -12136,7 +12151,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -12167,7 +12182,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -12198,7 +12213,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -12229,7 +12244,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -12260,7 +12275,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -12291,7 +12306,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -12322,7 +12337,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -12353,7 +12368,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -12384,7 +12399,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -12415,7 +12430,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -12446,7 +12461,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -12477,7 +12492,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -12508,7 +12523,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -13004,7 +13019,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -13035,7 +13050,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -13066,7 +13081,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -13097,7 +13112,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -13128,7 +13143,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -13159,7 +13174,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -13190,7 +13205,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -13221,7 +13236,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -13252,7 +13267,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -13283,7 +13298,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -13314,7 +13329,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -13345,7 +13360,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -13407,7 +13422,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel non moulu</t>
+          <t>Phosphate de chaux naturel</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -13650,7 +13665,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -13681,7 +13696,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -13712,7 +13727,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -13743,7 +13758,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -13774,7 +13789,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -13805,7 +13820,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -13836,7 +13851,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -13996,7 +14011,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -14027,7 +14042,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -14058,7 +14073,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -14089,7 +14104,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -14120,7 +14135,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -14151,7 +14166,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -14182,7 +14197,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -14213,7 +14228,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -14244,7 +14259,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -14275,7 +14290,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -14306,7 +14321,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -14337,7 +14352,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -14368,7 +14383,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -14399,7 +14414,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -14430,7 +14445,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -14461,7 +14476,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -14492,7 +14507,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -14523,7 +14538,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -14554,7 +14569,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -14585,7 +14600,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -14616,7 +14631,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -14647,7 +14662,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -14678,7 +14693,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -14709,7 +14724,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -14740,7 +14755,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -14771,7 +14786,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -14802,7 +14817,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -14833,7 +14848,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -14864,7 +14879,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -14895,7 +14910,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -14926,7 +14941,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -14957,7 +14972,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -15143,7 +15158,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -15174,7 +15189,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -15205,7 +15220,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -15236,7 +15251,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -16068,7 +16083,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -16099,7 +16114,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -16130,7 +16145,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -16161,7 +16176,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -16192,7 +16207,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -16223,7 +16238,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -16383,7 +16398,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -16414,7 +16429,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -16445,7 +16460,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -16476,7 +16491,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -16507,7 +16522,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -16538,7 +16553,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -16569,7 +16584,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -16600,7 +16615,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -16631,7 +16646,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -16662,7 +16677,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -16693,7 +16708,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -16724,7 +16739,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -16755,7 +16770,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -16786,7 +16801,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -16817,7 +16832,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -16848,7 +16863,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -16881,7 +16896,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -16912,7 +16927,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -16943,7 +16958,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Premium Zircon</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -16974,7 +16989,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -17005,7 +17020,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -17036,7 +17051,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -17067,7 +17082,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -17098,7 +17113,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -17129,7 +17144,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -17160,7 +17175,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -17191,7 +17206,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -17222,7 +17237,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -17253,7 +17268,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -17284,7 +17299,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -17315,7 +17330,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -17346,7 +17361,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Standard Zircon</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -17625,7 +17640,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -17656,7 +17671,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -17687,7 +17702,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -17718,7 +17733,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -17749,7 +17764,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -17780,7 +17795,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -18426,7 +18441,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -18457,7 +18472,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -18488,7 +18503,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -18519,7 +18534,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -18550,7 +18565,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>SOCOCIM INDUSTRIES</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -18710,7 +18725,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -18741,7 +18756,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -18772,7 +18787,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -18803,7 +18818,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -18834,7 +18849,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -18865,7 +18880,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -18896,7 +18911,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -18927,7 +18942,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -18958,7 +18973,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -18989,7 +19004,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -19020,7 +19035,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -19051,7 +19066,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -19082,7 +19097,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -19113,7 +19128,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -19144,7 +19159,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -19175,7 +19190,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -19206,7 +19221,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -19237,7 +19252,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -19268,7 +19283,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -19299,7 +19314,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -19330,7 +19345,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -19361,7 +19376,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -19392,7 +19407,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -19423,7 +19438,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -19454,7 +19469,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -19485,7 +19500,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -19516,7 +19531,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -19547,7 +19562,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -19578,7 +19593,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -19609,7 +19624,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -19640,7 +19655,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -19671,7 +19686,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -19702,7 +19717,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -19733,7 +19748,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -19764,7 +19779,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -19795,7 +19810,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -19826,7 +19841,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -19857,7 +19872,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -19888,7 +19903,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -19919,7 +19934,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -19950,7 +19965,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -19981,7 +19996,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -20012,7 +20027,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -20043,7 +20058,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -20074,7 +20089,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -20105,7 +20120,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -20136,7 +20151,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -20167,7 +20182,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -20198,7 +20213,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -20229,7 +20244,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -20260,7 +20275,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -22926,7 +22941,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>ATTAPULGITE</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
@@ -22957,7 +22972,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE ET ACIDES POLYPHOSPHORIQUES</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
@@ -22988,7 +23003,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE ET ACIDES POLYPHOSPHORIQUES</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -23019,7 +23034,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>ACIDE PHOSPHORIQUE ET ACIDES POLYPHOSPHORIQUES</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
@@ -23050,7 +23065,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
@@ -23081,7 +23096,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -23112,7 +23127,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
@@ -23143,7 +23158,7 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
@@ -23174,7 +23189,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
@@ -23205,7 +23220,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Engrais minéraux ou chimiques</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
@@ -23236,7 +23251,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Phosphate diammonique</t>
+          <t>DAP (Phosphate Diammonique)</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
@@ -23262,7 +23277,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -23293,7 +23308,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -23324,7 +23339,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -23355,7 +23370,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -23386,7 +23401,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -23515,7 +23530,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
@@ -23546,7 +23561,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -23577,7 +23592,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
@@ -23608,7 +23623,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
@@ -23639,7 +23654,7 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
@@ -23670,7 +23685,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
@@ -23701,7 +23716,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
@@ -23732,7 +23747,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
@@ -23763,7 +23778,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
@@ -24099,7 +24114,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -24130,7 +24145,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -24161,7 +24176,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -24192,7 +24207,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -24223,7 +24238,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -26827,7 +26842,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -26858,7 +26873,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -26889,7 +26904,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -28328,7 +28343,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>Acide Phosphorique 52%</t>
+          <t>Acide Phosphorique</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
@@ -28359,7 +28374,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
@@ -28390,7 +28405,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>Ilmenite 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -28540,7 +28555,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
@@ -28602,7 +28617,7 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
@@ -28633,7 +28648,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
@@ -28695,7 +28710,7 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
@@ -29568,7 +29583,7 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
@@ -29599,7 +29614,7 @@
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
@@ -29630,7 +29645,7 @@
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>Ilmenite 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
@@ -29687,7 +29702,7 @@
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>Sephos/G-PHOS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
@@ -29749,7 +29764,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>Sephos/G-PHOS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -29780,7 +29795,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>Sephos/G-PHOS</t>
+          <t>SEPHOS</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -29909,7 +29924,7 @@
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>Ilmenite 56</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
@@ -29940,7 +29955,7 @@
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
@@ -29971,7 +29986,7 @@
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
@@ -30002,7 +30017,7 @@
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D601" t="inlineStr">
@@ -30033,7 +30048,7 @@
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D602" t="inlineStr">
@@ -30064,7 +30079,7 @@
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D603" t="inlineStr">
@@ -30095,7 +30110,7 @@
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D604" t="inlineStr">
@@ -30126,7 +30141,7 @@
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D605" t="inlineStr">
@@ -30157,7 +30172,7 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D606" t="inlineStr">
@@ -30188,7 +30203,7 @@
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>Leucoxene</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D607" t="inlineStr">
@@ -30560,7 +30575,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>Attapulgide</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
@@ -30591,7 +30606,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>Attapulgide</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -30622,7 +30637,7 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>Attapulgide</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
@@ -30653,7 +30668,7 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Attapulgide</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
@@ -30834,7 +30849,7 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>Gécamines</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -30965,7 +30980,7 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>Gypsum</t>
+          <t>Gypse</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
@@ -30996,7 +31011,7 @@
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>Gypsum</t>
+          <t>Gypse</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
@@ -31365,7 +31380,7 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>Sococim</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -31427,7 +31442,7 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>Sococim</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -31520,7 +31535,7 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>Sococim</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
@@ -31582,7 +31597,7 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Sococim</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
@@ -31613,7 +31628,7 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Sococim</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
@@ -31649,7 +31664,7 @@
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
@@ -31990,7 +32005,7 @@
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
@@ -32021,7 +32036,7 @@
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
@@ -32052,7 +32067,7 @@
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
@@ -32269,7 +32284,7 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
@@ -32300,7 +32315,7 @@
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
@@ -32331,7 +32346,7 @@
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>MEDIUM GRADE ZIRCON SAND</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
@@ -32421,7 +32436,7 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>GECAMINE</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
@@ -32490,7 +32505,7 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>ILMENITE 56</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
@@ -32609,7 +32624,7 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>Sococim</t>
+          <t>SOCOCIM</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
@@ -33544,7 +33559,7 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>PHOSPHATE MONO AMMONIQUE</t>
+          <t>Phosphate Mono Ammonique</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -33575,7 +33590,7 @@
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>PHOSPHATE MONO AMMONIQUE</t>
+          <t>Phosphate Mono Ammonique</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
@@ -33606,7 +33621,7 @@
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>PHOSPHATE MONO AMMONIQUE</t>
+          <t>Phosphate Mono Ammonique</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
@@ -33637,7 +33652,7 @@
       </c>
       <c r="C718" t="inlineStr">
         <is>
-          <t>ILMENITE 54</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D718" t="inlineStr">
@@ -33668,7 +33683,7 @@
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>PHOSPHATE</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D719" t="inlineStr">
@@ -33699,7 +33714,7 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>NPK - Sac 50Kg</t>
+          <t>NPK</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
@@ -33730,7 +33745,7 @@
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>NPK - Sac 50Kg</t>
+          <t>NPK</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
@@ -33761,7 +33776,7 @@
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>Attapuglite</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D722" t="inlineStr">
@@ -33792,7 +33807,7 @@
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>Attapuglite</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
@@ -33823,7 +33838,7 @@
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>Attapuglite</t>
+          <t>Attapulgite</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
@@ -33849,12 +33864,12 @@
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>GECAMINE</t>
+          <t>GECAMINES</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
@@ -33885,7 +33900,7 @@
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
@@ -33918,7 +33933,7 @@
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>BASALTE</t>
+          <t>Basalte</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
@@ -33949,7 +33964,7 @@
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>ZIRCON MEDIUM</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
@@ -33980,7 +33995,7 @@
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>LEUCOXENE</t>
+          <t>Leucoxène</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
@@ -34011,7 +34026,7 @@
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>RUTILE</t>
+          <t>Rutile</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
@@ -34042,7 +34057,7 @@
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>ILMENITE 56</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
@@ -34073,7 +34088,7 @@
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>ZIRCON PREMIUM</t>
+          <t>Zircon Premium</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
@@ -34104,7 +34119,7 @@
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>ZIRCON STANDARD</t>
+          <t>Zircon Standard</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
@@ -34135,7 +34150,7 @@
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>ILMENITE 58</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
@@ -34166,7 +34181,7 @@
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>DAP - Sac 50Kg</t>
+          <t>DAP (Phosphate Diammonique)</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
@@ -34290,7 +34305,7 @@
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>DSP - Sac 50 Kg</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
@@ -34502,7 +34517,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -34533,7 +34548,7 @@
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
@@ -34564,7 +34579,7 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>Dangote</t>
+          <t>DANGOTE</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
@@ -35341,7 +35356,7 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>Talix Mines</t>
+          <t>TALIX</t>
         </is>
       </c>
       <c r="C773" t="inlineStr">
@@ -35377,7 +35392,7 @@
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Ilménite 54%</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D774" t="inlineStr">
@@ -35408,7 +35423,7 @@
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Ilménite 54%</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D775" t="inlineStr">
@@ -35439,7 +35454,7 @@
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Ilménite 54%</t>
+          <t>Ilménite 54</t>
         </is>
       </c>
       <c r="D776" t="inlineStr">
@@ -35470,7 +35485,7 @@
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>Ilménite 56%</t>
+          <t>Ilménite 56</t>
         </is>
       </c>
       <c r="D777" t="inlineStr">
@@ -35501,7 +35516,7 @@
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D778" t="inlineStr">
@@ -35534,7 +35549,7 @@
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D779" t="inlineStr">
@@ -35567,7 +35582,7 @@
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D780" t="inlineStr">
@@ -35598,7 +35613,7 @@
       </c>
       <c r="C781" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D781" t="inlineStr">
@@ -35629,7 +35644,7 @@
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>Ilménite 58%</t>
+          <t>Ilménite 58</t>
         </is>
       </c>
       <c r="D782" t="inlineStr">
@@ -36284,7 +36299,7 @@
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D803" t="inlineStr">
@@ -36315,7 +36330,7 @@
       </c>
       <c r="C804" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon</t>
+          <t>Medium Grade Zircon Sand</t>
         </is>
       </c>
       <c r="D804" t="inlineStr">
@@ -37090,7 +37105,7 @@
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>Autre</t>
+          <t>Autres</t>
         </is>
       </c>
       <c r="D829" t="inlineStr">
@@ -37121,7 +37136,7 @@
       </c>
       <c r="C830" t="inlineStr">
         <is>
-          <t>Autre</t>
+          <t>Autres</t>
         </is>
       </c>
       <c r="D830" t="inlineStr">

</xml_diff>

<commit_message>
Regroupe davantage les variantes de types de minerai
- Tous les grades de zircon (Premium, Standard, Medium Grade, Co-Product,
  Minerais de zirconium) fusionnés sous "Zircon".
- Grades d'Ilménite (54/56/58) fusionnés sous "Ilménite".
- Formes de Phosphate brut (Naturel, de chaux naturel, tricalcique, Sec
  Criblé, Rock Phosphate, alumino-calcique) fusionnées sous "Phosphate".
- "Minerais de titane"/"Titane" fusionnés sous "Titane".
- Conserve distincts les produits chimiques transformés (Acide
  Phosphorique, DAP, DSP, NPK, Phosphate Mono Ammonique, Engrais, Gypse).
- 36 types de minerai distincts au total (contre 50 après la première
  harmonisation, ~100 avant toute harmonisation).
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -657,7 +657,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel, ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%"). Ces variantes ont été harmonisées en un seul libellé par société et par minerai, pour permettre des tableaux croisés dynamiques fiables. Les libellés décrivant des grades ou produits réellement différents (ex : "Phosphate", "Phosphate Naturel", "Phosphate de chaux naturel", "Phosphate tricalcique", "Phosphate Sec Criblé") ont été conservés distincts, de même que les agrégats spécifiques à certaines années ("Minerais de titane", "Titane", "Sables minéralisés").</t>
+          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel, ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%"). Ces variantes ont été harmonisées en un seul libellé par société et par minerai, pour permettre des tableaux croisés dynamiques fiables. Les libellés décrivant des grades ou produits réellement différents (ex : "Phosphate", "Phosphate Naturel", "Phosphate de chaux naturel", "Phosphate tricalcique", "Phosphate Sec Criblé") ont été conservés distincts, de même que les agrégats spécifiques à certaines années ("Minerais de titane", "Titane", "Sables minéralisés"). Exception demandée : tous les grades de zircon ("Zircon Premium", "Zircon Standard", "Medium Grade Zircon Sand", "Zircon Co-Product", "Minerais de zirconium") ont été regroupés sous le seul libellé "Zircon", à la demande explicite . De même, les grades d'Ilménite (54/56/58), les formes de Phosphate (Naturel, de chaux naturel, tricalcique, Sec Criblé, Rock Phosphate, alumino-calcique) et les libellés de Titane ("Minerais de titane"/"Titane") ont été regroupés respectivement sous "Ilménite", "Phosphate" et "Titane". Restent distincts les produits chimiques transformés qui ne sont pas de simples grades de minerai brut : Acide Phosphorique, Acide Sulfurique, DAP, DSP, NPK, Phosphate Mono Ammonique, Engrais, Gypse.</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Phosphate Sec Criblé</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Phosphate alumino-calcique naturel non moulu</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Zircon Co-Product</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -6365,7 +6365,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -8212,7 +8212,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -8555,7 +8555,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -8617,7 +8617,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Phosphate Sec Criblé</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -9282,7 +9282,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -9313,7 +9313,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -9437,7 +9437,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -9592,7 +9592,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -9623,7 +9623,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Phosphate Sec Criblé</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -10612,7 +10612,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -10674,7 +10674,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -10705,7 +10705,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -10829,7 +10829,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Phosphate Sec Criblé</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -11903,7 +11903,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -11934,7 +11934,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -11996,7 +11996,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -12089,7 +12089,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -12120,7 +12120,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -12244,7 +12244,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -12306,7 +12306,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -12337,7 +12337,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -12461,7 +12461,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -12492,7 +12492,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -12523,7 +12523,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -13019,7 +13019,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -13050,7 +13050,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -13081,7 +13081,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -13112,7 +13112,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -13143,7 +13143,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -13174,7 +13174,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -13236,7 +13236,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -13267,7 +13267,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -13298,7 +13298,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Phosphate alumino-calcique naturel non moulu</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -14011,7 +14011,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -14042,7 +14042,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -14135,7 +14135,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -14166,7 +14166,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -14228,7 +14228,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -14290,7 +14290,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -14383,7 +14383,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -14414,7 +14414,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -14476,7 +14476,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -14507,7 +14507,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -14538,7 +14538,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -14569,7 +14569,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -14600,7 +14600,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -14631,7 +14631,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -14724,7 +14724,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -14786,7 +14786,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -14817,7 +14817,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -14848,7 +14848,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -14879,7 +14879,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -14910,7 +14910,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -14941,7 +14941,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -16398,7 +16398,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -16429,7 +16429,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -16460,7 +16460,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -16522,7 +16522,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -16553,7 +16553,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -16677,7 +16677,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -16708,7 +16708,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -16739,7 +16739,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -16801,7 +16801,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -16832,7 +16832,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -16863,7 +16863,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -16896,7 +16896,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -16958,7 +16958,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -16989,7 +16989,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -17020,7 +17020,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -17051,7 +17051,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -17082,7 +17082,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -17113,7 +17113,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -17144,7 +17144,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -17175,7 +17175,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -17206,7 +17206,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -17237,7 +17237,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -17299,7 +17299,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -17330,7 +17330,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -17361,7 +17361,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -17392,7 +17392,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Zircon Co-Product</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -17423,7 +17423,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Zircon Co-Product</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -18725,7 +18725,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -18756,7 +18756,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -18787,7 +18787,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -18818,7 +18818,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -18849,7 +18849,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -18880,7 +18880,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -18911,7 +18911,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -18942,7 +18942,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -18973,7 +18973,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -19004,7 +19004,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -19097,7 +19097,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -19159,7 +19159,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -19190,7 +19190,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -19221,7 +19221,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -19252,7 +19252,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -19314,7 +19314,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -19345,7 +19345,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -19376,7 +19376,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -19407,7 +19407,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -19438,7 +19438,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -19469,7 +19469,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -19500,7 +19500,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -19531,7 +19531,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -19562,7 +19562,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -19593,7 +19593,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -19624,7 +19624,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -19655,7 +19655,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -19686,7 +19686,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -19717,7 +19717,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -19748,7 +19748,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -19779,7 +19779,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -19810,7 +19810,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -19841,7 +19841,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -21267,7 +21267,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -21298,7 +21298,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -21329,7 +21329,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -21360,7 +21360,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -21391,7 +21391,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -21422,7 +21422,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -21484,7 +21484,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
@@ -21515,7 +21515,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -21546,7 +21546,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -21577,7 +21577,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -21608,7 +21608,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -21639,7 +21639,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -21670,7 +21670,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -21701,7 +21701,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -21732,7 +21732,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -21763,7 +21763,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -21794,7 +21794,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -21825,7 +21825,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -21856,7 +21856,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
@@ -21887,7 +21887,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
@@ -21918,7 +21918,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
@@ -21949,7 +21949,7 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
@@ -21980,7 +21980,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Minerais de zirconium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
@@ -22042,7 +22042,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -22073,7 +22073,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
@@ -22104,7 +22104,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -22135,7 +22135,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
@@ -22228,7 +22228,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -22259,7 +22259,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -22290,7 +22290,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
@@ -22321,7 +22321,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
@@ -22352,7 +22352,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
@@ -22383,7 +22383,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -22414,7 +22414,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -22445,7 +22445,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -22507,7 +22507,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -22538,7 +22538,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -22569,7 +22569,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
@@ -22600,7 +22600,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
@@ -22631,7 +22631,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -22662,7 +22662,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
@@ -22693,7 +22693,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -22724,7 +22724,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
@@ -22755,7 +22755,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
@@ -22786,7 +22786,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
@@ -22817,7 +22817,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -22848,7 +22848,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -22879,7 +22879,7 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -22910,7 +22910,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Minerais de titane</t>
+          <t>Titane</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -23437,7 +23437,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
@@ -23468,7 +23468,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
@@ -23499,7 +23499,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
@@ -28374,7 +28374,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
@@ -28405,7 +28405,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -28901,7 +28901,7 @@
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D565" t="inlineStr">
@@ -28932,7 +28932,7 @@
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">
@@ -28963,7 +28963,7 @@
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D567" t="inlineStr">
@@ -28994,7 +28994,7 @@
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
@@ -29025,7 +29025,7 @@
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
@@ -29056,7 +29056,7 @@
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D570" t="inlineStr">
@@ -29087,7 +29087,7 @@
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
@@ -29118,7 +29118,7 @@
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
@@ -29149,7 +29149,7 @@
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
@@ -29180,7 +29180,7 @@
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D574" t="inlineStr">
@@ -29211,7 +29211,7 @@
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
@@ -29242,7 +29242,7 @@
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
@@ -29273,7 +29273,7 @@
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D577" t="inlineStr">
@@ -29304,7 +29304,7 @@
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D578" t="inlineStr">
@@ -29335,7 +29335,7 @@
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D579" t="inlineStr">
@@ -29366,7 +29366,7 @@
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D581" t="inlineStr">
@@ -29428,7 +29428,7 @@
       </c>
       <c r="C582" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D582" t="inlineStr">
@@ -29459,7 +29459,7 @@
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D583" t="inlineStr">
@@ -29490,7 +29490,7 @@
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D584" t="inlineStr">
@@ -29521,7 +29521,7 @@
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D585" t="inlineStr">
@@ -29552,7 +29552,7 @@
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D586" t="inlineStr">
@@ -29583,7 +29583,7 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
@@ -29614,7 +29614,7 @@
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
@@ -29645,7 +29645,7 @@
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
@@ -29862,7 +29862,7 @@
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D596" t="inlineStr">
@@ -29893,7 +29893,7 @@
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">
@@ -29924,7 +29924,7 @@
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
@@ -31664,7 +31664,7 @@
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
@@ -32005,7 +32005,7 @@
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
@@ -32036,7 +32036,7 @@
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
@@ -32067,7 +32067,7 @@
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
@@ -32346,7 +32346,7 @@
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
@@ -32505,7 +32505,7 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
@@ -32753,7 +32753,7 @@
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>Rock Phosphate</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D705" t="inlineStr">
@@ -33280,7 +33280,7 @@
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
@@ -33311,7 +33311,7 @@
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D707" t="inlineStr">
@@ -33342,7 +33342,7 @@
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D708" t="inlineStr">
@@ -33373,7 +33373,7 @@
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D709" t="inlineStr">
@@ -33404,7 +33404,7 @@
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D710" t="inlineStr">
@@ -33435,7 +33435,7 @@
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D711" t="inlineStr">
@@ -33466,7 +33466,7 @@
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
@@ -33497,7 +33497,7 @@
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
@@ -33528,7 +33528,7 @@
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>Phosphate de chaux naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
@@ -33652,7 +33652,7 @@
       </c>
       <c r="C718" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D718" t="inlineStr">
@@ -33964,7 +33964,7 @@
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
@@ -34057,7 +34057,7 @@
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
@@ -34088,7 +34088,7 @@
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
@@ -34119,7 +34119,7 @@
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
@@ -34150,7 +34150,7 @@
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
@@ -34770,7 +34770,7 @@
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
@@ -34801,7 +34801,7 @@
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D755" t="inlineStr">
@@ -34832,7 +34832,7 @@
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D756" t="inlineStr">
@@ -34863,7 +34863,7 @@
       </c>
       <c r="C757" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D757" t="inlineStr">
@@ -34894,7 +34894,7 @@
       </c>
       <c r="C758" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D758" t="inlineStr">
@@ -34925,7 +34925,7 @@
       </c>
       <c r="C759" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D759" t="inlineStr">
@@ -34956,7 +34956,7 @@
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>Phosphate Naturel</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D760" t="inlineStr">
@@ -34987,7 +34987,7 @@
       </c>
       <c r="C761" t="inlineStr">
         <is>
-          <t>Phosphate tricalcique</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D761" t="inlineStr">
@@ -35018,7 +35018,7 @@
       </c>
       <c r="C762" t="inlineStr">
         <is>
-          <t>Phosphate tricalcique</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D762" t="inlineStr">
@@ -35049,7 +35049,7 @@
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>Phosphate tricalcique</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D763" t="inlineStr">
@@ -35080,7 +35080,7 @@
       </c>
       <c r="C764" t="inlineStr">
         <is>
-          <t>Phosphate tricalcique</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="D764" t="inlineStr">
@@ -35392,7 +35392,7 @@
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D774" t="inlineStr">
@@ -35423,7 +35423,7 @@
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D775" t="inlineStr">
@@ -35454,7 +35454,7 @@
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Ilménite 54</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D776" t="inlineStr">
@@ -35485,7 +35485,7 @@
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>Ilménite 56</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D777" t="inlineStr">
@@ -35516,7 +35516,7 @@
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D778" t="inlineStr">
@@ -35549,7 +35549,7 @@
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D779" t="inlineStr">
@@ -35582,7 +35582,7 @@
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D780" t="inlineStr">
@@ -35613,7 +35613,7 @@
       </c>
       <c r="C781" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D781" t="inlineStr">
@@ -35644,7 +35644,7 @@
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>Ilménite 58</t>
+          <t>Ilménite</t>
         </is>
       </c>
       <c r="D782" t="inlineStr">
@@ -35954,7 +35954,7 @@
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D792" t="inlineStr">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D793" t="inlineStr">
@@ -36016,7 +36016,7 @@
       </c>
       <c r="C794" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D794" t="inlineStr">
@@ -36047,7 +36047,7 @@
       </c>
       <c r="C795" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D795" t="inlineStr">
@@ -36080,7 +36080,7 @@
       </c>
       <c r="C796" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D796" t="inlineStr">
@@ -36111,7 +36111,7 @@
       </c>
       <c r="C797" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D797" t="inlineStr">
@@ -36142,7 +36142,7 @@
       </c>
       <c r="C798" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D798" t="inlineStr">
@@ -36173,7 +36173,7 @@
       </c>
       <c r="C799" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D799" t="inlineStr">
@@ -36204,7 +36204,7 @@
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D800" t="inlineStr">
@@ -36235,7 +36235,7 @@
       </c>
       <c r="C801" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D801" t="inlineStr">
@@ -36268,7 +36268,7 @@
       </c>
       <c r="C802" t="inlineStr">
         <is>
-          <t>Zircon Standard</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D802" t="inlineStr">
@@ -36299,7 +36299,7 @@
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D803" t="inlineStr">
@@ -36330,7 +36330,7 @@
       </c>
       <c r="C804" t="inlineStr">
         <is>
-          <t>Medium Grade Zircon Sand</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D804" t="inlineStr">
@@ -36361,7 +36361,7 @@
       </c>
       <c r="C805" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D805" t="inlineStr">
@@ -36392,7 +36392,7 @@
       </c>
       <c r="C806" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D806" t="inlineStr">
@@ -36423,7 +36423,7 @@
       </c>
       <c r="C807" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D807" t="inlineStr">
@@ -36454,7 +36454,7 @@
       </c>
       <c r="C808" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D808" t="inlineStr">
@@ -36485,7 +36485,7 @@
       </c>
       <c r="C809" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D809" t="inlineStr">
@@ -36516,7 +36516,7 @@
       </c>
       <c r="C810" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D810" t="inlineStr">
@@ -36547,7 +36547,7 @@
       </c>
       <c r="C811" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D811" t="inlineStr">
@@ -36578,7 +36578,7 @@
       </c>
       <c r="C812" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D812" t="inlineStr">
@@ -36609,7 +36609,7 @@
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D813" t="inlineStr">
@@ -36640,7 +36640,7 @@
       </c>
       <c r="C814" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D814" t="inlineStr">
@@ -36671,7 +36671,7 @@
       </c>
       <c r="C815" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D815" t="inlineStr">
@@ -36702,7 +36702,7 @@
       </c>
       <c r="C816" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D816" t="inlineStr">
@@ -36733,7 +36733,7 @@
       </c>
       <c r="C817" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D817" t="inlineStr">
@@ -36764,7 +36764,7 @@
       </c>
       <c r="C818" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D818" t="inlineStr">
@@ -36795,7 +36795,7 @@
       </c>
       <c r="C819" t="inlineStr">
         <is>
-          <t>Zircon Premium</t>
+          <t>Zircon</t>
         </is>
       </c>
       <c r="D819" t="inlineStr">

</xml_diff>

<commit_message>
Regroupe les produits engrais (DAP, DSP, NPK, Phosphate Mono Ammonique)
Fusionne DAP, DSP, NPK et Phosphate Mono Ammonique sous "Engrais",
suivant la même logique que les regroupements précédents. Restent
distincts les acides industriels (Acide Phosphorique, Acide Sulfurique)
et le Gypse, qui ne sont pas des engrais. 32 types de minerai distincts
au total.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -657,7 +657,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel, ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%"). Ces variantes ont été harmonisées en un seul libellé par société et par minerai, pour permettre des tableaux croisés dynamiques fiables. Les libellés décrivant des grades ou produits réellement différents (ex : "Phosphate", "Phosphate Naturel", "Phosphate de chaux naturel", "Phosphate tricalcique", "Phosphate Sec Criblé") ont été conservés distincts, de même que les agrégats spécifiques à certaines années ("Minerais de titane", "Titane", "Sables minéralisés"). Exception demandée : tous les grades de zircon ("Zircon Premium", "Zircon Standard", "Medium Grade Zircon Sand", "Zircon Co-Product", "Minerais de zirconium") ont été regroupés sous le seul libellé "Zircon", à la demande explicite . De même, les grades d'Ilménite (54/56/58), les formes de Phosphate (Naturel, de chaux naturel, tricalcique, Sec Criblé, Rock Phosphate, alumino-calcique) et les libellés de Titane ("Minerais de titane"/"Titane") ont été regroupés respectivement sous "Ilménite", "Phosphate" et "Titane". Restent distincts les produits chimiques transformés qui ne sont pas de simples grades de minerai brut : Acide Phosphorique, Acide Sulfurique, DAP, DSP, NPK, Phosphate Mono Ammonique, Engrais, Gypse.</t>
+          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel, ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%"). Ces variantes ont été harmonisées en un seul libellé par société et par minerai, pour permettre des tableaux croisés dynamiques fiables. Les libellés décrivant des grades ou produits réellement différents (ex : "Phosphate", "Phosphate Naturel", "Phosphate de chaux naturel", "Phosphate tricalcique", "Phosphate Sec Criblé") ont été conservés distincts, de même que les agrégats spécifiques à certaines années ("Minerais de titane", "Titane", "Sables minéralisés"). Exception demandée : tous les grades de zircon ("Zircon Premium", "Zircon Standard", "Medium Grade Zircon Sand", "Zircon Co-Product", "Minerais de zirconium") ont été regroupés sous le seul libellé "Zircon", à la demande explicite . De même, les grades d'Ilménite (54/56/58), les formes de Phosphate (Naturel, de chaux naturel, tricalcique, Sec Criblé, Rock Phosphate, alumino-calcique) et les libellés de Titane ("Minerais de titane"/"Titane") ont été regroupés respectivement sous "Ilménite", "Phosphate" et "Titane". Les produits finis de type engrais (DAP, DSP, NPK, Phosphate Mono Ammonique) ont également été regroupés sous "Engrais". Restent distincts les acides industriels (Acide Phosphorique, Acide Sulfurique) et le Gypse, qui ne sont pas des engrais.</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4772,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>DAP (Phosphate Diammonique)</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -23251,7 +23251,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>DAP (Phosphate Diammonique)</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
@@ -30699,7 +30699,7 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D623" t="inlineStr">
@@ -30730,7 +30730,7 @@
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
@@ -30761,7 +30761,7 @@
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
@@ -30792,7 +30792,7 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>NPK</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
@@ -30823,7 +30823,7 @@
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>NPK</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
@@ -32098,7 +32098,7 @@
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>NPK</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
@@ -32129,7 +32129,7 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>NPK</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
@@ -32598,7 +32598,7 @@
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
@@ -33559,7 +33559,7 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>Phosphate Mono Ammonique</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -33590,7 +33590,7 @@
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>Phosphate Mono Ammonique</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
@@ -33621,7 +33621,7 @@
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>Phosphate Mono Ammonique</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
@@ -33714,7 +33714,7 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>NPK</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
@@ -33745,7 +33745,7 @@
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>NPK</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
@@ -34181,7 +34181,7 @@
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>DAP (Phosphate Diammonique)</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
@@ -34305,7 +34305,7 @@
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Engrais</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">

</xml_diff>

<commit_message>
Réécrit la feuille Notes pour refléter l'état final de l'harmonisation
Remplace le texte accumulé par petites modifications successives (devenu
incohérent) par une version propre et structurée : sources par année,
conventions de codage, et un récapitulatif clair des regroupements de
types de minerai (Zircon, Ilménite, Titane, Phosphate, Engrais) avec ce
qui reste distinct et pourquoi.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -497,6 +497,9 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -511,6 +514,9 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -538,7 +544,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Tableaux "Détail des productions du secteur minier" et "Détail des exportations et ventes locales du secteur minier" des rapports ITIE Sénégal 2019-2021 (numérotation Tableau 32/33 selon les années).</t>
+          <t>Tableaux "Détail des productions du secteur minier" et "Détail des exportations et ventes locales du secteur minier" des rapports ITIE Sénégal 2019-2021 (numérotation Tableau 32/33 selon les années). Le tableau des exportations 2021 était initialement tronqué dans l'extrait PDF fourni (il manquait la fin du Leucoxène, le Zircon, le Rutile et la catégorie "Autre") ; la page manquante a été fournie séparément et intégrée.</t>
         </is>
       </c>
     </row>
@@ -578,6 +584,9 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -617,7 +626,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Toutes les cellules des colonnes Quantité et Valeur sont des nombres purs (aucun texte tel que "USD" ou "*" mélangé à la valeur). Sur la feuille "production", certaines valeurs de production (GCO 2014-2016, notamment) sont exprimées en dollars US dans le rapport source plutôt qu'en FCFA : une colonne "Devise" a été ajoutée (G) pour l'indiquer explicitement ("FCFA" ou "USD") au lieu de convertir arbitrairement ou de laisser "USD" en texte dans la valeur. Les valeurs suivies d'un astérisque dans le rapport 2014 (SOSECAR, COGECA, SODEVIT) signifient "valeur calculée sur la base de la valeur marchande déclarée par la société" ; l'astérisque a été retiré du nombre et cette précision ajoutée en commentaire de cellule.</t>
+          <t>Toutes les cellules des colonnes Quantité et Valeur sont des nombres purs (aucun texte tel que "USD" ou "*" mélangé à la valeur). Certaines valeurs de production (GCO 2014-2016, notamment) sont exprimées en dollars US dans le rapport source plutôt qu'en FCFA, sans conversion de taux de change : une colonne "Devise" indique explicitement "FCFA" ou "USD" pour chaque ligne. Les valeurs suivies d'un astérisque dans le rapport 2014 (SOSECAR, COGECA, SODEVIT) signifient "valeur calculée sur la base de la valeur marchande déclarée par la société" ; l'astérisque a été retiré du nombre et cette précision ajoutée en commentaire de cellule.</t>
         </is>
       </c>
     </row>
@@ -633,31 +642,109 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Note : exportations 2021 (complétées)</t>
+          <t>Harmonisation des noms de sociétés et de types de minerai</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Le fichier source 2021.pdf initialement fourni (extrait de 5 pages) était tronqué : il manquait une page du Tableau 33 (fin du Leucoxène, Zircon Standard, Medium Grade Zircon, Zircon Premium, Rutile, et la catégorie "Autre"/SOCOCIM). Cette page manquante a été fournie séparément et intégrée à la feuille exportation. Les lignes de totaux par substance et le total général du tableau source n'ont pas été reportés (seules les lignes détaillées par opérateur/pays figurent dans la feuille).</t>
+          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel — ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "DANGOTE" / "Dangote", "GECAMINES" / "GECAMINE" / "Gécamines"). Ces variantes ont systématiquement été unifiées en un seul libellé par société.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pour les types de minerai, les variantes de casse/orthographe/accents d'un même produit ont été unifiées (ex : "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%", "Attapulgite" / "Attapulgide" / "Attapuglite"). Au-delà de cette unification orthographique, à la demande explicite, les différents grades/formes d'une même famille de minerai ont aussi été regroupés sous un seul libellé, y compris lorsque le rapport source les distinguait :</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Harmonisation des noms de sociétés et de types de minerai</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Zircon</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Regroupe Zircon Premium, Zircon Standard, Medium Grade Zircon Sand, Zircon Co-Product, Minerais de zirconium, Zircon.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel, ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "Ilmenite 54" / "ILMENITE 54" / "Ilménite 54%"). Ces variantes ont été harmonisées en un seul libellé par société et par minerai, pour permettre des tableaux croisés dynamiques fiables. Les libellés décrivant des grades ou produits réellement différents (ex : "Phosphate", "Phosphate Naturel", "Phosphate de chaux naturel", "Phosphate tricalcique", "Phosphate Sec Criblé") ont été conservés distincts, de même que les agrégats spécifiques à certaines années ("Minerais de titane", "Titane", "Sables minéralisés"). Exception demandée : tous les grades de zircon ("Zircon Premium", "Zircon Standard", "Medium Grade Zircon Sand", "Zircon Co-Product", "Minerais de zirconium") ont été regroupés sous le seul libellé "Zircon", à la demande explicite . De même, les grades d'Ilménite (54/56/58), les formes de Phosphate (Naturel, de chaux naturel, tricalcique, Sec Criblé, Rock Phosphate, alumino-calcique) et les libellés de Titane ("Minerais de titane"/"Titane") ont été regroupés respectivement sous "Ilménite", "Phosphate" et "Titane". Les produits finis de type engrais (DAP, DSP, NPK, Phosphate Mono Ammonique) ont également été regroupés sous "Engrais". Restent distincts les acides industriels (Acide Phosphorique, Acide Sulfurique) et le Gypse, qui ne sont pas des engrais.</t>
+          <t>Ilménite</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Regroupe Ilménite 54, Ilménite 56, Ilménite 58.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Titane</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Regroupe Minerais de titane, Titane.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Phosphate</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Regroupe Phosphate, Phosphate Naturel, Phosphate de chaux naturel, Phosphate tricalcique, Phosphate Sec Criblé, Rock Phosphate, Phosphate alumino-calcique naturel non moulu (grades/formes de minerai de phosphate brut).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Engrais</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Regroupe Engrais, DAP (Phosphate Diammonique), DSP, NPK, Phosphate Mono Ammonique (produits finis de type engrais).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Restent distincts</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Acide Phosphorique, Acide Sulfurique et Gypse (produits chimiques industriels, pas des grades de minerai brut ni des engrais), ainsi que "Sables minéralisés" (agrégat d'exportation regroupant plusieurs minerais GCO, propre à certaines années, non assimilable à un seul minerai).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Après harmonisation complète : 22 sociétés distinctes et 32 types de minerai distincts sur les deux feuilles (contre respectivement 30 et une centaine de variantes avant harmonisation).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retire les couleurs de fond et le tiret long dans la feuille Notes
Supprime le remplissage coloré des en-têtes de section (Notes) et
remplace le tiret cadratin (—) par un tiret simple, pour un rendu plus
sobre et des caractères standards.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -62,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -76,6 +76,9 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,11 +500,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Portée</t>
         </is>
@@ -514,11 +515,9 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Sources par année</t>
         </is>
@@ -584,11 +583,9 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Conventions et codes utilisés</t>
         </is>
@@ -642,11 +639,9 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
+    <row r="18"/>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Harmonisation des noms de sociétés et de types de minerai</t>
         </is>
@@ -655,7 +650,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel — ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "DANGOTE" / "Dangote", "GECAMINES" / "GECAMINE" / "Gécamines"). Ces variantes ont systématiquement été unifiées en un seul libellé par société.</t>
+          <t>Les rapports sources orthographient parfois différemment une même société ou un même minerai selon l'année (majuscules, accents, singulier/pluriel - ex : "SOCOCIM" / "SOCOCIM INDUSTRIES", "DANGOTE" / "Dangote", "GECAMINES" / "GECAMINE" / "Gécamines"). Ces variantes ont systématiquement été unifiées en un seul libellé par société.</t>
         </is>
       </c>
     </row>
@@ -738,9 +733,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Harmonise les unités de volume/poids et documente les facteurs de conversion
- Minerais bruts (hors Or/Argent) : convertis vers Tonne (Kg/1000, MT
  renommé en Tonne).
- Or et Argent : convertis vers Once troy (1 once = 31,1034768 g),
  qu'ils soient initialement en Kg, Gramme ou Tonne.
- Mètre cube conservé tel quel (pas de conversion en Tonne, densité du
  matériau inconnue).
- Corrige une erreur du rapport source 2018 : l'unité "Tonne" indiquée
  pour l'Or/Argent de PMC (production et exportation) était physiquement
  impossible (156 925 tonnes d'or) ; les quantités correspondent en
  réalité à des onces troy, corrigées sans changer la valeur numérique.
- Documente tous les facteurs de conversion et cette correction dans la
  feuille Notes.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.####"/>
+    <numFmt numFmtId="165" formatCode="#,##0.######"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -62,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -79,6 +80,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -486,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -500,7 +502,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -515,7 +516,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -583,7 +583,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -639,7 +638,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
@@ -733,11 +731,72 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Après harmonisation complète : 22 sociétés distinctes et 32 types de minerai distincts sur les deux feuilles (contre respectivement 30 et une centaine de variantes avant harmonisation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Harmonisation des unités de volume/poids</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Les rapports sources expriment les quantités dans des unités différentes selon les années (Tonne, Kg, Gramme, MT, Once/Onces/Ounce, M3/Mètre cube...). Toutes les quantités ont été converties vers une seule unité par famille de minerai :</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Minerais bruts / matériaux (tout sauf Or et Argent)</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Unité cible : Tonne. Conversions : 1 Tonne = 1 000 Kg (Kg divisé par 1 000) ; "MT" (Metric Tonne) = Tonne (renommage, aucune conversion nécessaire).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Or et Argent</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Unité cible : Once (once troy). Conversion utilisée : 1 once troy = 31,1034768 grammes (valeur standard internationale). Kg converti en once via les grammes (Kg × 1 000 / 31,1034768) ; Gramme converti directement (Gramme / 31,1034768) ; Tonne convertie en once (Tonne × 1 000 000 / 31,1034768, soit environ × 32 150,7466).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Volumes (Mètre cube)</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Les quantités en M3/m3/Mètre cube n'ont PAS été converties en Tonne (densité du matériau inconnue et variable, une conversion aurait été arbitraire) ; seules les variantes orthographiques ont été unifiées sous "Mètre cube".</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Correction signalée : PMC Or/Argent 2018</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Le rapport ITIE 2018 indique par erreur l'unité "Tonne" pour la production ET l'exportation d'Or et d'Argent de PMC (156 925,68 "Tonnes" d'or et 10 114,22 "Tonnes" d'argent en production ; 143 389,00 et 9 323,50 en exportation), ce qui est physiquement impossible (156 925 tonnes d'or dépasseraient largement tout l'or jamais extrait dans le monde). Les quantités elles-mêmes sont cohérentes avec des onces troy (ordre de grandeur et valeur en FCFA/once compatibles avec le cours de l'or/argent de 2018 et avec la production de PMC les autres années). Ces 4 cellules ont donc été considérées comme des "Onces" mal étiquetées "Tonne" dans le rapport source, et l'unité a été corrigée en conséquence SANS multiplier la quantité (elle était déjà exprimée en onces).</t>
         </is>
       </c>
     </row>
@@ -913,7 +972,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
@@ -944,7 +1003,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1615,7 +1674,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
@@ -1708,7 +1767,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
@@ -1770,7 +1829,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
@@ -1801,7 +1860,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2470,7 +2529,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
@@ -2567,7 +2626,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
@@ -2629,7 +2688,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
@@ -2660,7 +2719,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3331,7 +3390,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
@@ -3364,7 +3423,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
@@ -3397,7 +3456,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
@@ -3461,7 +3520,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
@@ -4248,7 +4307,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E110" s="4" t="n">
@@ -4279,7 +4338,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E111" s="4" t="n">
@@ -4341,7 +4400,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E113" s="4" t="n">
@@ -4471,7 +4530,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E117" s="5" t="n">
@@ -4502,7 +4561,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E118" s="5" t="n">
@@ -5117,7 +5176,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E137" s="4" t="n">
@@ -5148,7 +5207,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E138" s="4" t="n">
@@ -5210,7 +5269,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E140" s="4" t="n">
@@ -5241,7 +5300,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E141" s="5" t="n">
@@ -5272,7 +5331,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E142" s="5" t="n">
@@ -5303,7 +5362,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E143" s="4" t="n">
@@ -5334,7 +5393,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E144" s="4" t="n">
@@ -5365,7 +5424,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E145" s="4" t="n">
@@ -5396,7 +5455,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E146" s="4" t="n">
@@ -5427,7 +5486,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E147" s="4" t="n">
@@ -5458,7 +5517,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E148" s="4" t="n">
@@ -5489,7 +5548,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E149" s="4" t="n">
@@ -5520,7 +5579,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E150" s="4" t="n">
@@ -5551,7 +5610,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E151" s="4" t="n">
@@ -5582,7 +5641,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E152" s="4" t="n">
@@ -5613,7 +5672,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E153" s="4" t="n">
@@ -5644,7 +5703,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E154" s="4" t="n">
@@ -5675,7 +5734,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E155" s="4" t="n">
@@ -5706,7 +5765,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E156" s="4" t="n">
@@ -5737,7 +5796,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E157" s="4" t="n">
@@ -5768,7 +5827,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E158" s="4" t="n">
@@ -5799,7 +5858,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E159" s="4" t="n">
@@ -5830,7 +5889,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E160" s="4" t="n">
@@ -5861,7 +5920,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E161" s="4" t="n">
@@ -5892,7 +5951,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E162" s="4" t="n">
@@ -5923,7 +5982,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E163" s="4" t="n">
@@ -5954,7 +6013,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E164" s="4" t="n">
@@ -5985,7 +6044,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E165" s="4" t="n">
@@ -6016,7 +6075,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E166" s="4" t="n">
@@ -6047,7 +6106,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E167" s="4" t="n">
@@ -6078,7 +6137,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E168" s="4" t="n">
@@ -6109,7 +6168,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E169" s="4" t="n">
@@ -6140,7 +6199,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E170" s="4" t="n">
@@ -6171,7 +6230,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E171" s="4" t="n">
@@ -6202,7 +6261,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E172" s="4" t="n">
@@ -6233,11 +6292,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Tonnes</t>
-        </is>
-      </c>
-      <c r="E173" s="4" t="n">
-        <v>7</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="n">
+        <v>225055.226</v>
       </c>
       <c r="F173" s="4" t="n">
         <v>217680000000</v>
@@ -6264,11 +6323,11 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E174" s="5" t="n">
-        <v>5.8</v>
+        <v>186474.3301</v>
       </c>
       <c r="F174" s="4" t="n">
         <v>179340000000</v>
@@ -6295,7 +6354,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E175" s="5" t="n">
@@ -6326,7 +6385,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E176" s="5" t="n">
@@ -6357,7 +6416,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E177" s="5" t="n">
@@ -6388,7 +6447,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E178" s="5" t="n">
@@ -6419,7 +6478,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E179" s="5" t="n">
@@ -6450,7 +6509,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E180" s="5" t="n">
@@ -6481,7 +6540,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E181" s="4" t="n">
@@ -6512,7 +6571,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E182" s="4" t="n">
@@ -6543,7 +6602,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E183" s="4" t="n">
@@ -6574,7 +6633,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E184" s="5" t="n">
@@ -6605,7 +6664,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E185" s="4" t="n">
@@ -6636,7 +6695,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E186" s="5" t="n">
@@ -6667,7 +6726,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E187" s="4" t="n">
@@ -6698,7 +6757,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E188" s="4" t="n">
@@ -6729,7 +6788,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E189" s="4" t="n">
@@ -6760,7 +6819,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E190" s="4" t="n">
@@ -6822,7 +6881,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E192" s="4" t="n">
@@ -6853,7 +6912,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E193" s="4" t="n">
@@ -6886,7 +6945,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E194" s="4" t="n">
@@ -7016,11 +7075,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E198" s="5" t="n">
-        <v>12.2</v>
+        <v>392239.1081</v>
       </c>
       <c r="F198" s="4" t="n">
         <v>390697165834</v>
@@ -7047,11 +7106,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Tonnes</t>
-        </is>
-      </c>
-      <c r="E199" s="4" t="n">
-        <v>1</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="n">
+        <v>32150.7466</v>
       </c>
       <c r="F199" s="4" t="n">
         <v>453360287</v>
@@ -7078,11 +7137,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Tonnes</t>
-        </is>
-      </c>
-      <c r="E200" s="4" t="n">
-        <v>4</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E200" s="5" t="n">
+        <v>128602.9863</v>
       </c>
       <c r="F200" t="inlineStr">
         <is>
@@ -7111,11 +7170,11 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E201" s="5" t="n">
-        <v>0.3</v>
+        <v>9645.224</v>
       </c>
       <c r="F201" s="4" t="n">
         <v>130156827</v>
@@ -7952,11 +8011,11 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>TONNE</t>
-        </is>
-      </c>
-      <c r="E228" s="4" t="n">
-        <v>11</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E228" s="5" t="n">
+        <v>353658.2123</v>
       </c>
       <c r="F228" s="4" t="n">
         <v>393709507828</v>
@@ -7983,11 +8042,11 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E229" s="5" t="n">
-        <v>4.0255</v>
+        <v>129422.8303</v>
       </c>
       <c r="F229" s="4" t="n">
         <v>145989168041</v>
@@ -8014,11 +8073,11 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E230" s="5" t="n">
-        <v>0.0485</v>
+        <v>1559.3112</v>
       </c>
       <c r="F230" t="inlineStr">
         <is>
@@ -8047,7 +8106,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E231" s="4" t="n">
@@ -8078,7 +8137,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E232" s="4" t="n">
@@ -8109,7 +8168,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E233" s="4" t="n">
@@ -8140,7 +8199,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E234" s="4" t="n">
@@ -8171,7 +8230,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E235" s="4" t="n">
@@ -8202,7 +8261,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E236" s="4" t="n">
@@ -8233,7 +8292,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E237" s="4" t="n">
@@ -8297,7 +8356,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E239" s="4" t="n">
@@ -8328,7 +8387,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E240" s="4" t="n">
@@ -8359,7 +8418,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E241" s="4" t="n">
@@ -8390,7 +8449,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E242" s="4" t="n">
@@ -8421,7 +8480,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E243" s="4" t="n">
@@ -8452,7 +8511,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E244" s="4" t="n">
@@ -8483,7 +8542,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>METRE CUBE</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E245" s="4" t="n">
@@ -8514,7 +8573,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E246" s="4" t="n">
@@ -8545,7 +8604,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E247" s="4" t="n">
@@ -8576,7 +8635,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E248" s="4" t="n">
@@ -8607,7 +8666,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E249" s="4" t="n">
@@ -8640,7 +8699,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E250" s="4" t="n">
@@ -8671,7 +8730,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E251" s="4" t="n">
@@ -8702,7 +8761,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E252" s="4" t="n">
@@ -8733,7 +8792,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E253" s="4" t="n">
@@ -8764,7 +8823,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E254" s="4" t="n">
@@ -8795,7 +8854,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E255" s="4" t="n">
@@ -8826,11 +8885,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>TONNE</t>
-        </is>
-      </c>
-      <c r="E256" s="4" t="n">
-        <v>1</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E256" s="5" t="n">
+        <v>32150.7466</v>
       </c>
       <c r="F256" s="4" t="n">
         <v>382666065</v>
@@ -8857,11 +8916,11 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E257" s="5" t="n">
-        <v>0.3254</v>
+        <v>10461.8529</v>
       </c>
       <c r="F257" s="4" t="n">
         <v>142020334</v>
@@ -8888,7 +8947,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E258" s="4" t="n">
@@ -8919,7 +8978,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E259" s="4" t="n">
@@ -8952,7 +9011,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E260" s="4" t="n">
@@ -8985,7 +9044,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E261" s="4" t="n">
@@ -9018,7 +9077,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Onces troy (Oz)</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E262" s="4" t="n">
@@ -9049,7 +9108,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Onces troy (Oz)</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E263" s="4" t="n">
@@ -9080,7 +9139,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E264" s="4" t="n">
@@ -9111,7 +9170,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E265" s="4" t="n">
@@ -9142,7 +9201,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E266" s="4" t="n">
@@ -9175,7 +9234,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E267" s="4" t="n">
@@ -9208,7 +9267,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E268" s="4" t="n">
@@ -9241,7 +9300,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E269" s="4" t="n">
@@ -9336,7 +9395,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E272" s="4" t="n">
@@ -9367,7 +9426,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E273" s="4" t="n">
@@ -9398,7 +9457,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E274" s="4" t="n">
@@ -9429,7 +9488,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E275" s="4" t="n">
@@ -9460,7 +9519,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E276" s="4" t="n">
@@ -9491,7 +9550,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E277" s="4" t="n">
@@ -9522,7 +9581,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E278" s="4" t="n">
@@ -9553,7 +9612,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E279" s="4" t="n">
@@ -9584,7 +9643,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E280" s="4" t="n">
@@ -9615,7 +9674,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E281" s="4" t="n">
@@ -9646,7 +9705,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E282" s="4" t="n">
@@ -9677,7 +9736,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E283" s="4" t="n">
@@ -9708,7 +9767,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E284" s="4" t="n">
@@ -9739,7 +9798,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E285" s="4" t="n">
@@ -9770,7 +9829,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E286" s="4" t="n">
@@ -9801,7 +9860,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E287" s="4" t="n">
@@ -9865,7 +9924,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E289" s="4" t="n">
@@ -9898,7 +9957,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E290" s="4" t="n">
@@ -9931,7 +9990,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E291" s="4" t="n">
@@ -9964,7 +10023,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E292" s="4" t="n">
@@ -9997,7 +10056,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>mètre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E293" s="4" t="n">
@@ -10030,7 +10089,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E294" s="4" t="n">
@@ -10063,7 +10122,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E295" s="4" t="n">
@@ -10096,7 +10155,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E296" s="4" t="n">
@@ -10129,7 +10188,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E297" s="4" t="n">
@@ -10162,7 +10221,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E298" s="4" t="n">
@@ -10195,7 +10254,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E299" s="4" t="n">
@@ -10228,11 +10287,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Gramme</t>
-        </is>
-      </c>
-      <c r="E300" s="4" t="n">
-        <v>55883</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E300" s="5" t="n">
+        <v>1796.6802</v>
       </c>
       <c r="F300" t="inlineStr">
         <is>
@@ -10261,11 +10320,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Gramme</t>
-        </is>
-      </c>
-      <c r="E301" s="4" t="n">
-        <v>2999</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E301" s="5" t="n">
+        <v>96.42010000000001</v>
       </c>
       <c r="F301" t="inlineStr">
         <is>
@@ -10294,7 +10353,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E302" s="4" t="n">
@@ -10325,7 +10384,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E303" s="4" t="n">
@@ -10356,7 +10415,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E304" s="4" t="n">
@@ -10387,7 +10446,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Onces troy (Oz)</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E305" s="4" t="n">
@@ -10418,7 +10477,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Onces troy (Oz)</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E306" s="4" t="n">
@@ -10449,7 +10508,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E307" s="4" t="n">
@@ -10480,7 +10539,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E308" s="4" t="n">
@@ -10511,7 +10570,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E309" s="4" t="n">
@@ -10542,7 +10601,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E310" s="4" t="n">
@@ -10573,7 +10632,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E311" s="4" t="n">
@@ -10604,7 +10663,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E312" s="4" t="n">
@@ -10635,7 +10694,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E313" s="4" t="n">
@@ -10666,7 +10725,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E314" s="4" t="n">
@@ -10697,7 +10756,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E315" s="4" t="n">
@@ -10728,7 +10787,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E316" s="4" t="n">
@@ -10759,7 +10818,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E317" s="4" t="n">
@@ -10790,7 +10849,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E318" s="4" t="n">
@@ -10821,7 +10880,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E319" s="4" t="n">
@@ -10852,7 +10911,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E320" s="4" t="n">
@@ -10883,7 +10942,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E321" s="4" t="n">
@@ -10914,7 +10973,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E322" s="4" t="n">
@@ -10945,7 +11004,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Onces troy (Oz)</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E323" s="4" t="n">
@@ -10976,7 +11035,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E324" s="4" t="n">
@@ -11007,7 +11066,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E325" s="4" t="n">
@@ -11038,7 +11097,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>TONNES</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E326" s="4" t="n">
@@ -11069,7 +11128,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>TONNES</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E327" s="4" t="n">
@@ -11133,7 +11192,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E329" s="4" t="n">
@@ -11166,7 +11225,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E330" s="4" t="n">
@@ -11199,7 +11258,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E331" s="4" t="n">
@@ -11232,7 +11291,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E332" s="4" t="n">
@@ -11265,7 +11324,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>METRE CUBE</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E333" s="4" t="n">
@@ -11298,7 +11357,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>TONNES</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E334" s="4" t="n">
@@ -11331,7 +11390,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>TONNES</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E335" s="4" t="n">
@@ -11364,7 +11423,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E336" s="4" t="n">
@@ -11397,11 +11456,11 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>GRAMME</t>
-        </is>
-      </c>
-      <c r="E337" s="4" t="n">
-        <v>51536</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E337" s="5" t="n">
+        <v>1656.9209</v>
       </c>
       <c r="F337" t="inlineStr">
         <is>
@@ -11430,7 +11489,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E338" s="4" t="n">
@@ -11771,7 +11830,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
@@ -11802,7 +11861,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
@@ -13600,7 +13659,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
@@ -13724,7 +13783,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Métre cube</t>
+          <t>Mètre cube</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
@@ -13972,7 +14031,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
@@ -14003,7 +14062,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
@@ -16359,7 +16418,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E158" s="4" t="n">
@@ -16390,7 +16449,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Ounce</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E159" s="4" t="n">
@@ -21228,7 +21287,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E315" s="5" t="n">
@@ -21259,7 +21318,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E316" s="5" t="n">
@@ -23894,10 +23953,10 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Tonne</t>
-        </is>
-      </c>
-      <c r="E401" s="4" t="n">
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E401" s="5" t="n">
         <v>143389</v>
       </c>
       <c r="F401" s="4" t="n">
@@ -23925,7 +23984,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Tonne</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E402" s="5" t="n">
@@ -23956,11 +24015,11 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E403" s="4" t="n">
-        <v>300000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E403" s="8" t="n">
+        <v>300</v>
       </c>
       <c r="F403" s="4" t="n">
         <v>2550000</v>
@@ -23987,11 +24046,11 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E404" s="4" t="n">
-        <v>229</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E404" s="8" t="n">
+        <v>0.229</v>
       </c>
       <c r="F404" s="4" t="n">
         <v>196786</v>
@@ -24018,11 +24077,11 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E405" s="4" t="n">
-        <v>64610000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E405" s="8" t="n">
+        <v>64610</v>
       </c>
       <c r="F405" s="4" t="n">
         <v>534230281</v>
@@ -24049,11 +24108,11 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E406" s="4" t="n">
-        <v>86870800</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E406" s="8" t="n">
+        <v>86870.8</v>
       </c>
       <c r="F406" s="4" t="n">
         <v>3572174000</v>
@@ -24080,11 +24139,11 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E407" s="4" t="n">
-        <v>700000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E407" s="8" t="n">
+        <v>700</v>
       </c>
       <c r="F407" s="4" t="n">
         <v>26950000</v>
@@ -24111,11 +24170,11 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E408" s="4" t="n">
-        <v>697800</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E408" s="8" t="n">
+        <v>697.8</v>
       </c>
       <c r="F408" s="4" t="n">
         <v>35509500</v>
@@ -24142,11 +24201,11 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E409" s="4" t="n">
-        <v>873956700</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E409" s="8" t="n">
+        <v>873956.7</v>
       </c>
       <c r="F409" s="4" t="n">
         <v>37783173175</v>
@@ -24173,11 +24232,11 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E410" s="4" t="n">
-        <v>3000000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E410" s="8" t="n">
+        <v>3000</v>
       </c>
       <c r="F410" s="4" t="n">
         <v>121000000</v>
@@ -24204,11 +24263,11 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E411" s="4" t="n">
-        <v>15168040</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E411" s="8" t="n">
+        <v>15168.04</v>
       </c>
       <c r="F411" s="4" t="n">
         <v>583132600</v>
@@ -24235,11 +24294,11 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E412" s="4" t="n">
-        <v>280000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E412" s="8" t="n">
+        <v>280</v>
       </c>
       <c r="F412" s="4" t="n">
         <v>10920000</v>
@@ -24266,11 +24325,11 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E413" s="4" t="n">
-        <v>15122000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E413" s="8" t="n">
+        <v>15122</v>
       </c>
       <c r="F413" s="4" t="n">
         <v>593149480</v>
@@ -24297,11 +24356,11 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E414" s="4" t="n">
-        <v>411969000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E414" s="8" t="n">
+        <v>411969</v>
       </c>
       <c r="F414" s="4" t="n">
         <v>16042005860</v>
@@ -24328,11 +24387,11 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E415" s="4" t="n">
-        <v>1000000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E415" s="8" t="n">
+        <v>1000</v>
       </c>
       <c r="F415" s="4" t="n">
         <v>30825600</v>
@@ -24359,11 +24418,11 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E416" s="4" t="n">
-        <v>35000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E416" s="8" t="n">
+        <v>35</v>
       </c>
       <c r="F416" s="4" t="n">
         <v>1400000</v>
@@ -24390,11 +24449,11 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E417" s="4" t="n">
-        <v>25699730</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E417" s="8" t="n">
+        <v>25699.73</v>
       </c>
       <c r="F417" s="4" t="n">
         <v>1122957948</v>
@@ -24421,11 +24480,11 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E418" s="4" t="n">
-        <v>790000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E418" s="8" t="n">
+        <v>790</v>
       </c>
       <c r="F418" s="4" t="n">
         <v>31600000</v>
@@ -24452,11 +24511,11 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E419" s="4" t="n">
-        <v>5256000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E419" s="8" t="n">
+        <v>5256</v>
       </c>
       <c r="F419" s="4" t="n">
         <v>282330000</v>
@@ -24483,11 +24542,11 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E420" s="4" t="n">
-        <v>309554000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E420" s="8" t="n">
+        <v>309554</v>
       </c>
       <c r="F420" s="4" t="n">
         <v>13294733480</v>
@@ -24514,11 +24573,11 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E421" s="4" t="n">
-        <v>3716000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E421" s="8" t="n">
+        <v>3716</v>
       </c>
       <c r="F421" s="4" t="n">
         <v>148640000</v>
@@ -24545,11 +24604,11 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E422" s="4" t="n">
-        <v>6221</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E422" s="5" t="n">
+        <v>200009.7944</v>
       </c>
       <c r="F422" s="4" t="n">
         <v>151885748355</v>
@@ -24576,11 +24635,11 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E423" s="4" t="n">
-        <v>7845</v>
+          <t>Once</t>
+        </is>
+      </c>
+      <c r="E423" s="5" t="n">
+        <v>252222.6068</v>
       </c>
       <c r="F423" s="4" t="n">
         <v>189853050512</v>
@@ -24607,11 +24666,11 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E424" s="4" t="n">
-        <v>38807328</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E424" s="8" t="n">
+        <v>38807.328</v>
       </c>
       <c r="F424" s="4" t="n">
         <v>1053061182</v>
@@ -24638,11 +24697,11 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E425" s="4" t="n">
-        <v>540000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E425" s="8" t="n">
+        <v>540</v>
       </c>
       <c r="F425" s="4" t="n">
         <v>33635941</v>
@@ -24669,11 +24728,11 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E426" s="4" t="n">
-        <v>600000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E426" s="8" t="n">
+        <v>600</v>
       </c>
       <c r="F426" s="4" t="n">
         <v>46009041</v>
@@ -24700,11 +24759,11 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E427" s="4" t="n">
-        <v>6306365</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E427" s="8" t="n">
+        <v>6306.365</v>
       </c>
       <c r="F427" s="4" t="n">
         <v>177601263</v>
@@ -24731,11 +24790,11 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E428" s="4" t="n">
-        <v>2214000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E428" s="8" t="n">
+        <v>2214</v>
       </c>
       <c r="F428" s="4" t="n">
         <v>167689729</v>
@@ -24762,11 +24821,11 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E429" s="4" t="n">
-        <v>325000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E429" s="8" t="n">
+        <v>325</v>
       </c>
       <c r="F429" s="4" t="n">
         <v>22390853</v>
@@ -24793,11 +24852,11 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E430" s="4" t="n">
-        <v>5504281</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E430" s="8" t="n">
+        <v>5504.281</v>
       </c>
       <c r="F430" s="4" t="n">
         <v>237885351</v>
@@ -24824,11 +24883,11 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E431" s="4" t="n">
-        <v>206661472</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E431" s="8" t="n">
+        <v>206661.472</v>
       </c>
       <c r="F431" s="4" t="n">
         <v>8590562499</v>
@@ -24855,11 +24914,11 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E432" s="4" t="n">
-        <v>48349124</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E432" s="8" t="n">
+        <v>48349.124</v>
       </c>
       <c r="F432" s="4" t="n">
         <v>1996738634</v>
@@ -24886,11 +24945,11 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E433" s="4" t="n">
-        <v>1028934</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E433" s="8" t="n">
+        <v>1028.934</v>
       </c>
       <c r="F433" s="4" t="n">
         <v>49020084</v>
@@ -24917,11 +24976,11 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E434" s="4" t="n">
-        <v>51053338</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E434" s="8" t="n">
+        <v>51053.338</v>
       </c>
       <c r="F434" s="4" t="n">
         <v>1009154057</v>
@@ -24948,11 +25007,11 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E435" s="4" t="n">
-        <v>225802469</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E435" s="8" t="n">
+        <v>225802.469</v>
       </c>
       <c r="F435" s="4" t="n">
         <v>8947306557</v>
@@ -24979,11 +25038,11 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E436" s="4" t="n">
-        <v>2043</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E436" s="8" t="n">
+        <v>2.043</v>
       </c>
       <c r="F436" s="4" t="n">
         <v>4662145</v>
@@ -25010,11 +25069,11 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E437" s="4" t="n">
-        <v>439920</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E437" s="8" t="n">
+        <v>439.92</v>
       </c>
       <c r="F437" s="4" t="n">
         <v>175825218</v>
@@ -25041,11 +25100,11 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E438" s="4" t="n">
-        <v>35755440</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E438" s="8" t="n">
+        <v>35755.44</v>
       </c>
       <c r="F438" s="4" t="n">
         <v>3277431091</v>
@@ -25072,11 +25131,11 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E439" s="4" t="n">
-        <v>50251475</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E439" s="8" t="n">
+        <v>50251.475</v>
       </c>
       <c r="F439" s="4" t="n">
         <v>6509347684</v>
@@ -25103,11 +25162,11 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E440" s="4" t="n">
-        <v>1060034</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E440" s="8" t="n">
+        <v>1060.034</v>
       </c>
       <c r="F440" s="4" t="n">
         <v>586821696</v>
@@ -25134,11 +25193,11 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E441" s="4" t="n">
-        <v>640000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E441" s="8" t="n">
+        <v>640</v>
       </c>
       <c r="F441" s="4" t="n">
         <v>348132720</v>
@@ -25165,11 +25224,11 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E442" s="4" t="n">
-        <v>740000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E442" s="8" t="n">
+        <v>740</v>
       </c>
       <c r="F442" s="4" t="n">
         <v>323447690</v>
@@ -25196,11 +25255,11 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E443" s="4" t="n">
-        <v>360000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E443" s="8" t="n">
+        <v>360</v>
       </c>
       <c r="F443" s="4" t="n">
         <v>204683877</v>
@@ -25227,11 +25286,11 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E444" s="4" t="n">
-        <v>131972632</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E444" s="8" t="n">
+        <v>131972.632</v>
       </c>
       <c r="F444" s="4" t="n">
         <v>13887462924</v>
@@ -25258,11 +25317,11 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E445" s="4" t="n">
-        <v>33003612</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E445" s="8" t="n">
+        <v>33003.612</v>
       </c>
       <c r="F445" s="4" t="n">
         <v>2822576820</v>
@@ -25289,11 +25348,11 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E446" s="4" t="n">
-        <v>120000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E446" s="8" t="n">
+        <v>120</v>
       </c>
       <c r="F446" s="4" t="n">
         <v>76506597</v>
@@ -25320,11 +25379,11 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E447" s="4" t="n">
-        <v>1560000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E447" s="8" t="n">
+        <v>1560</v>
       </c>
       <c r="F447" s="4" t="n">
         <v>666909876</v>
@@ -25351,11 +25410,11 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E448" s="4" t="n">
-        <v>10720864</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E448" s="8" t="n">
+        <v>10720.864</v>
       </c>
       <c r="F448" s="4" t="n">
         <v>1620371391</v>
@@ -25382,11 +25441,11 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E449" s="4" t="n">
-        <v>120000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E449" s="8" t="n">
+        <v>120</v>
       </c>
       <c r="F449" s="4" t="n">
         <v>50574672</v>
@@ -25413,11 +25472,11 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E450" s="4" t="n">
-        <v>60000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E450" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="F450" s="4" t="n">
         <v>25579584</v>
@@ -25444,11 +25503,11 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E451" s="4" t="n">
-        <v>12000173</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E451" s="8" t="n">
+        <v>12000.173</v>
       </c>
       <c r="F451" s="4" t="n">
         <v>1477074834</v>
@@ -25475,11 +25534,11 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E452" s="4" t="n">
-        <v>137096702</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E452" s="8" t="n">
+        <v>137096.702</v>
       </c>
       <c r="F452" s="4" t="n">
         <v>11805065457</v>
@@ -25506,11 +25565,11 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E453" s="4" t="n">
-        <v>440000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E453" s="8" t="n">
+        <v>440</v>
       </c>
       <c r="F453" s="4" t="n">
         <v>204756900</v>
@@ -25537,11 +25596,11 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E454" s="4" t="n">
-        <v>32689506</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E454" s="8" t="n">
+        <v>32689.506</v>
       </c>
       <c r="F454" s="4" t="n">
         <v>2859546469</v>
@@ -25568,11 +25627,11 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E455" s="4" t="n">
-        <v>34515169</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E455" s="8" t="n">
+        <v>34515.169</v>
       </c>
       <c r="F455" s="4" t="n">
         <v>3040784148</v>
@@ -25599,11 +25658,11 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E456" s="4" t="n">
-        <v>60016</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E456" s="8" t="n">
+        <v>60.016</v>
       </c>
       <c r="F456" s="4" t="n">
         <v>24846360</v>
@@ -25630,11 +25689,11 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E457" s="4" t="n">
-        <v>35678434</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E457" s="8" t="n">
+        <v>35678.434</v>
       </c>
       <c r="F457" s="4" t="n">
         <v>3037501898</v>
@@ -25661,11 +25720,11 @@
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E458" s="4" t="n">
-        <v>16268802</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E458" s="8" t="n">
+        <v>16268.802</v>
       </c>
       <c r="F458" s="4" t="n">
         <v>2114063389</v>
@@ -25692,11 +25751,11 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E459" s="4" t="n">
-        <v>400000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E459" s="8" t="n">
+        <v>400</v>
       </c>
       <c r="F459" s="4" t="n">
         <v>169857630</v>
@@ -25723,11 +25782,11 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E460" s="4" t="n">
-        <v>20000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E460" s="8" t="n">
+        <v>20</v>
       </c>
       <c r="F460" s="4" t="n">
         <v>13712600</v>
@@ -25754,11 +25813,11 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E461" s="4" t="n">
-        <v>60000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E461" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="F461" s="4" t="n">
         <v>25934856</v>
@@ -25785,11 +25844,11 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E462" s="4" t="n">
-        <v>793020</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E462" s="8" t="n">
+        <v>793.02</v>
       </c>
       <c r="F462" s="4" t="n">
         <v>697609772</v>
@@ -25816,11 +25875,11 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E463" s="4" t="n">
-        <v>1509951</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E463" s="8" t="n">
+        <v>1509.951</v>
       </c>
       <c r="F463" s="4" t="n">
         <v>1510675462</v>
@@ -25847,11 +25906,11 @@
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E464" s="4" t="n">
-        <v>3545219</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E464" s="8" t="n">
+        <v>3545.219</v>
       </c>
       <c r="F464" s="4" t="n">
         <v>3132088193</v>
@@ -25878,11 +25937,11 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E465" s="4" t="n">
-        <v>432590</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E465" s="8" t="n">
+        <v>432.59</v>
       </c>
       <c r="F465" s="4" t="n">
         <v>407332695</v>
@@ -25909,11 +25968,11 @@
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E466" s="4" t="n">
-        <v>18211958</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E466" s="8" t="n">
+        <v>18211.958</v>
       </c>
       <c r="F466" s="4" t="n">
         <v>9588818298</v>
@@ -25940,11 +25999,11 @@
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E467" s="4" t="n">
-        <v>480000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E467" s="8" t="n">
+        <v>480</v>
       </c>
       <c r="F467" s="4" t="n">
         <v>287176700</v>
@@ -25971,11 +26030,11 @@
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E468" s="4" t="n">
-        <v>200000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E468" s="8" t="n">
+        <v>200</v>
       </c>
       <c r="F468" s="4" t="n">
         <v>125996450</v>
@@ -26002,11 +26061,11 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E469" s="4" t="n">
-        <v>18835030</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E469" s="8" t="n">
+        <v>18835.03</v>
       </c>
       <c r="F469" s="4" t="n">
         <v>16759043528</v>
@@ -26033,11 +26092,11 @@
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E470" s="4" t="n">
-        <v>5856480</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E470" s="8" t="n">
+        <v>5856.48</v>
       </c>
       <c r="F470" s="4" t="n">
         <v>5698452377</v>
@@ -26064,11 +26123,11 @@
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E471" s="4" t="n">
-        <v>1883970</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E471" s="8" t="n">
+        <v>1883.97</v>
       </c>
       <c r="F471" s="4" t="n">
         <v>1768991238</v>
@@ -26095,11 +26154,11 @@
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E472" s="4" t="n">
-        <v>1005884</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E472" s="8" t="n">
+        <v>1005.884</v>
       </c>
       <c r="F472" s="4" t="n">
         <v>235791515</v>
@@ -26126,11 +26185,11 @@
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E473" s="4" t="n">
-        <v>787563</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E473" s="8" t="n">
+        <v>787.563</v>
       </c>
       <c r="F473" s="4" t="n">
         <v>697884692</v>
@@ -26157,11 +26216,11 @@
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E474" s="4" t="n">
-        <v>3019409</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E474" s="8" t="n">
+        <v>3019.409</v>
       </c>
       <c r="F474" s="4" t="n">
         <v>2752054212</v>
@@ -26188,11 +26247,11 @@
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E475" s="4" t="n">
-        <v>3581186</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E475" s="8" t="n">
+        <v>3581.186</v>
       </c>
       <c r="F475" s="4" t="n">
         <v>3487715930</v>
@@ -26219,11 +26278,11 @@
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E476" s="4" t="n">
-        <v>300946</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E476" s="8" t="n">
+        <v>300.946</v>
       </c>
       <c r="F476" s="4" t="n">
         <v>280903277</v>
@@ -26250,11 +26309,11 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E477" s="4" t="n">
-        <v>692353</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E477" s="8" t="n">
+        <v>692.353</v>
       </c>
       <c r="F477" s="4" t="n">
         <v>1318614759</v>
@@ -26281,11 +26340,11 @@
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E478" s="4" t="n">
-        <v>881772</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E478" s="8" t="n">
+        <v>881.772</v>
       </c>
       <c r="F478" s="4" t="n">
         <v>819992836</v>
@@ -26312,11 +26371,11 @@
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E479" s="4" t="n">
-        <v>1742801</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E479" s="8" t="n">
+        <v>1742.801</v>
       </c>
       <c r="F479" s="4" t="n">
         <v>1510053148</v>
@@ -26343,11 +26402,11 @@
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E480" s="4" t="n">
-        <v>529819</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E480" s="8" t="n">
+        <v>529.819</v>
       </c>
       <c r="F480" s="4" t="n">
         <v>622824529</v>
@@ -26374,11 +26433,11 @@
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E481" s="4" t="n">
-        <v>59114</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E481" s="8" t="n">
+        <v>59.114</v>
       </c>
       <c r="F481" s="4" t="n">
         <v>54513959</v>
@@ -26405,11 +26464,11 @@
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E482" s="4" t="n">
-        <v>22610453</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E482" s="8" t="n">
+        <v>22610.453</v>
       </c>
       <c r="F482" s="4" t="n">
         <v>7952913239</v>
@@ -26436,11 +26495,11 @@
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E483" s="4" t="n">
-        <v>1652912</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E483" s="8" t="n">
+        <v>1652.912</v>
       </c>
       <c r="F483" s="4" t="n">
         <v>1458268587</v>
@@ -26467,11 +26526,11 @@
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E484" s="4" t="n">
-        <v>60000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E484" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="F484" s="4" t="n">
         <v>24394860</v>
@@ -26498,11 +26557,11 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="E485" s="4" t="n">
-        <v>40013</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E485" s="8" t="n">
+        <v>40.013</v>
       </c>
       <c r="F485" s="4" t="n">
         <v>32994042</v>
@@ -28335,11 +28394,11 @@
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E544" s="5" t="n">
-        <v>10.5416</v>
+        <v>338920.31</v>
       </c>
       <c r="F544" s="4" t="n">
         <v>380045730082</v>
@@ -28366,11 +28425,11 @@
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E545" s="5" t="n">
-        <v>4.0319</v>
+        <v>129628.5951</v>
       </c>
       <c r="F545" s="4" t="n">
         <v>147954684761</v>
@@ -28397,11 +28456,11 @@
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E546" s="5" t="n">
-        <v>0.3485</v>
+        <v>11204.5352</v>
       </c>
       <c r="F546" s="4" t="n">
         <v>12540974385</v>
@@ -28428,7 +28487,7 @@
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E547" s="4" t="n">
@@ -28459,7 +28518,7 @@
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E548" s="4" t="n">
@@ -28490,7 +28549,7 @@
       </c>
       <c r="D549" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E549" s="4" t="n">
@@ -28521,7 +28580,7 @@
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E550" s="4" t="n">
@@ -28552,7 +28611,7 @@
       </c>
       <c r="D551" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E551" s="4" t="n">
@@ -28583,7 +28642,7 @@
       </c>
       <c r="D552" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E552" s="4" t="n">
@@ -28614,7 +28673,7 @@
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E553" s="4" t="n">
@@ -28645,7 +28704,7 @@
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E554" s="4" t="n">
@@ -28676,7 +28735,7 @@
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E555" s="4" t="n">
@@ -28707,7 +28766,7 @@
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E556" s="4" t="n">
@@ -28738,7 +28797,7 @@
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E557" s="4" t="n">
@@ -28769,7 +28828,7 @@
       </c>
       <c r="D558" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E558" s="4" t="n">
@@ -28800,7 +28859,7 @@
       </c>
       <c r="D559" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E559" s="4" t="n">
@@ -28831,7 +28890,7 @@
       </c>
       <c r="D560" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E560" s="4" t="n">
@@ -28862,7 +28921,7 @@
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E561" s="4" t="n">
@@ -28893,7 +28952,7 @@
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E562" s="4" t="n">
@@ -28924,7 +28983,7 @@
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E563" s="4" t="n">
@@ -28955,7 +29014,7 @@
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E564" s="4" t="n">
@@ -28986,7 +29045,7 @@
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E565" s="4" t="n">
@@ -29017,7 +29076,7 @@
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E566" s="4" t="n">
@@ -29048,7 +29107,7 @@
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E567" s="4" t="n">
@@ -29079,7 +29138,7 @@
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E568" s="4" t="n">
@@ -29110,7 +29169,7 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E569" s="4" t="n">
@@ -29141,7 +29200,7 @@
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E570" s="4" t="n">
@@ -29172,7 +29231,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E571" s="4" t="n">
@@ -29203,7 +29262,7 @@
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E572" s="4" t="n">
@@ -29234,7 +29293,7 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E573" s="4" t="n">
@@ -29265,7 +29324,7 @@
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E574" s="4" t="n">
@@ -29296,7 +29355,7 @@
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E575" s="4" t="n">
@@ -29327,7 +29386,7 @@
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E576" s="4" t="n">
@@ -29358,7 +29417,7 @@
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E577" s="4" t="n">
@@ -29389,7 +29448,7 @@
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E578" s="4" t="n">
@@ -29420,7 +29479,7 @@
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E579" s="4" t="n">
@@ -29451,7 +29510,7 @@
       </c>
       <c r="D580" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E580" s="4" t="n">
@@ -29482,7 +29541,7 @@
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E581" s="4" t="n">
@@ -29513,7 +29572,7 @@
       </c>
       <c r="D582" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E582" s="4" t="n">
@@ -29544,7 +29603,7 @@
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E583" s="4" t="n">
@@ -29575,7 +29634,7 @@
       </c>
       <c r="D584" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E584" s="4" t="n">
@@ -29606,7 +29665,7 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E585" s="4" t="n">
@@ -29637,7 +29696,7 @@
       </c>
       <c r="D586" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E586" s="4" t="n">
@@ -29668,7 +29727,7 @@
       </c>
       <c r="D587" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E587" s="4" t="n">
@@ -29699,7 +29758,7 @@
       </c>
       <c r="D588" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E588" s="4" t="n">
@@ -29730,7 +29789,7 @@
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E589" s="4" t="n">
@@ -29761,7 +29820,7 @@
       </c>
       <c r="D590" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E590" s="4" t="n">
@@ -29792,7 +29851,7 @@
       </c>
       <c r="D591" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E591" s="4" t="n">
@@ -29823,7 +29882,7 @@
       </c>
       <c r="D592" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E592" s="4" t="n">
@@ -29854,7 +29913,7 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E593" s="4" t="n">
@@ -29885,7 +29944,7 @@
       </c>
       <c r="D594" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E594" s="4" t="n">
@@ -29916,7 +29975,7 @@
       </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E595" s="4" t="n">
@@ -29947,7 +30006,7 @@
       </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E596" s="4" t="n">
@@ -29978,7 +30037,7 @@
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E597" s="4" t="n">
@@ -30009,7 +30068,7 @@
       </c>
       <c r="D598" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E598" s="4" t="n">
@@ -30040,7 +30099,7 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E599" s="4" t="n">
@@ -30071,7 +30130,7 @@
       </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E600" s="4" t="n">
@@ -30102,7 +30161,7 @@
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E601" s="4" t="n">
@@ -30133,7 +30192,7 @@
       </c>
       <c r="D602" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E602" s="4" t="n">
@@ -30164,7 +30223,7 @@
       </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E603" s="4" t="n">
@@ -30195,7 +30254,7 @@
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E604" s="4" t="n">
@@ -30226,7 +30285,7 @@
       </c>
       <c r="D605" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E605" s="4" t="n">
@@ -30257,7 +30316,7 @@
       </c>
       <c r="D606" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E606" s="4" t="n">
@@ -30288,7 +30347,7 @@
       </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E607" s="4" t="n">
@@ -30319,7 +30378,7 @@
       </c>
       <c r="D608" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E608" s="4" t="n">
@@ -30350,7 +30409,7 @@
       </c>
       <c r="D609" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E609" s="4" t="n">
@@ -30381,7 +30440,7 @@
       </c>
       <c r="D610" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E610" s="4" t="n">
@@ -30412,7 +30471,7 @@
       </c>
       <c r="D611" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E611" s="4" t="n">
@@ -30443,7 +30502,7 @@
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E612" s="4" t="n">
@@ -30474,7 +30533,7 @@
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E613" s="4" t="n">
@@ -30505,7 +30564,7 @@
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E614" s="4" t="n">
@@ -30536,7 +30595,7 @@
       </c>
       <c r="D615" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E615" s="4" t="n">
@@ -30567,7 +30626,7 @@
       </c>
       <c r="D616" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E616" s="4" t="n">
@@ -30598,7 +30657,7 @@
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E617" s="4" t="n">
@@ -30629,7 +30688,7 @@
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E618" s="4" t="n">
@@ -30660,7 +30719,7 @@
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E619" s="4" t="n">
@@ -30691,7 +30750,7 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E620" s="4" t="n">
@@ -30722,7 +30781,7 @@
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E621" s="4" t="n">
@@ -30753,7 +30812,7 @@
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E622" s="4" t="n">
@@ -30784,7 +30843,7 @@
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E623" s="4" t="n">
@@ -30815,7 +30874,7 @@
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E624" s="4" t="n">
@@ -30846,7 +30905,7 @@
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E625" s="4" t="n">
@@ -30877,7 +30936,7 @@
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E626" s="4" t="n">
@@ -30908,7 +30967,7 @@
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E627" s="4" t="n">
@@ -30939,7 +30998,7 @@
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
@@ -30972,7 +31031,7 @@
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E629" s="4" t="n">
@@ -31003,7 +31062,7 @@
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E630" s="4" t="n">
@@ -31034,7 +31093,7 @@
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E631" s="4" t="n">
@@ -31065,7 +31124,7 @@
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E632" s="4" t="n">
@@ -31096,7 +31155,7 @@
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E633" s="4" t="n">
@@ -31160,7 +31219,7 @@
       </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E635" s="4" t="n">
@@ -31191,7 +31250,7 @@
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E636" s="4" t="n">
@@ -31253,7 +31312,7 @@
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E638" s="4" t="n">
@@ -31284,7 +31343,7 @@
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E639" s="4" t="n">
@@ -31315,7 +31374,7 @@
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E640" s="4" t="n">
@@ -31346,7 +31405,7 @@
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E641" s="4" t="n">
@@ -31377,7 +31436,7 @@
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E642" s="4" t="n">
@@ -31408,7 +31467,7 @@
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E643" s="4" t="n">
@@ -31470,7 +31529,7 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E645" s="4" t="n">
@@ -31532,7 +31591,7 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E647" s="4" t="n">
@@ -31563,7 +31622,7 @@
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E648" s="4" t="n">
@@ -31625,7 +31684,7 @@
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E650" s="4" t="n">
@@ -31656,7 +31715,7 @@
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E651" s="4" t="n">
@@ -31687,7 +31746,7 @@
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E652" s="4" t="n">
@@ -31718,7 +31777,7 @@
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E653" s="4" t="n">
@@ -31749,7 +31808,7 @@
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E654" s="4" t="n">
@@ -31842,7 +31901,7 @@
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E657" s="4" t="n">
@@ -31997,7 +32056,7 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E662" s="4" t="n">
@@ -32028,7 +32087,7 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E663" s="4" t="n">
@@ -32059,7 +32118,7 @@
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E664" s="4" t="n">
@@ -32090,7 +32149,7 @@
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E665" s="4" t="n">
@@ -32121,7 +32180,7 @@
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E666" s="4" t="n">
@@ -32152,7 +32211,7 @@
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E667" s="4" t="n">
@@ -32183,7 +32242,7 @@
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E668" s="4" t="n">
@@ -32214,7 +32273,7 @@
       </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E669" s="4" t="n">
@@ -32245,7 +32304,7 @@
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E670" s="4" t="n">
@@ -32276,7 +32335,7 @@
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E671" s="4" t="n">
@@ -32307,7 +32366,7 @@
       </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E672" s="4" t="n">
@@ -32338,7 +32397,7 @@
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E673" s="4" t="n">
@@ -32369,7 +32428,7 @@
       </c>
       <c r="D674" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E674" s="4" t="n">
@@ -32400,7 +32459,7 @@
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E675" s="4" t="n">
@@ -32431,7 +32490,7 @@
       </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E676" s="4" t="n">
@@ -32462,7 +32521,7 @@
       </c>
       <c r="D677" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E677" s="4" t="n">
@@ -32493,7 +32552,7 @@
       </c>
       <c r="D678" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
@@ -32557,7 +32616,7 @@
       </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E680" t="inlineStr">
@@ -32590,7 +32649,7 @@
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E681" s="4" t="n">
@@ -32621,7 +32680,7 @@
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E682" s="4" t="n">
@@ -32683,7 +32742,7 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E684" s="4" t="n">
@@ -32714,7 +32773,7 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>TONNE</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E685" s="4" t="n">
@@ -32745,7 +32804,7 @@
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E686" s="4" t="n">
@@ -32776,7 +32835,7 @@
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E687" s="4" t="n">
@@ -32807,7 +32866,7 @@
       </c>
       <c r="D688" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E688" s="4" t="n">
@@ -32838,7 +32897,7 @@
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E689" s="4" t="n">
@@ -32869,7 +32928,7 @@
       </c>
       <c r="D690" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E690" s="4" t="n">
@@ -32900,7 +32959,7 @@
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E691" s="4" t="n">
@@ -32931,7 +32990,7 @@
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E692" s="4" t="n">
@@ -32962,7 +33021,7 @@
       </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E693" s="4" t="n">
@@ -32993,7 +33052,7 @@
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E694" s="4" t="n">
@@ -33644,7 +33703,7 @@
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E715" s="4" t="n">
@@ -33675,7 +33734,7 @@
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E716" s="4" t="n">
@@ -33706,7 +33765,7 @@
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E717" s="4" t="n">
@@ -33799,7 +33858,7 @@
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E720" s="4" t="n">
@@ -33830,7 +33889,7 @@
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E721" s="4" t="n">
@@ -34266,7 +34325,7 @@
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E735" s="4" t="n">
@@ -34297,7 +34356,7 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E736" s="4" t="n">
@@ -34328,7 +34387,7 @@
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E737" s="4" t="n">
@@ -34359,7 +34418,7 @@
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E738" s="4" t="n">
@@ -34390,7 +34449,7 @@
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E739" s="4" t="n">
@@ -34421,7 +34480,7 @@
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E740" s="4" t="n">
@@ -34452,7 +34511,7 @@
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E741" s="4" t="n">
@@ -34483,7 +34542,7 @@
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E742" s="4" t="n">
@@ -34514,7 +34573,7 @@
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Onces</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="E743" s="4" t="n">

</xml_diff>

<commit_message>
Harmonise les pays de destination dans la feuille exportation
Unifie les variantes de langue/casse/orthographe d'un même pays (ex :
China/CHINE/Chine, Germany/ALLEMAGNE, Ukranie/Ukraine, Switzerland/
Suisse, Dubai/Émirats Arabes Unis) sous un libellé canonique en français.
Conserve distincts les agrégats régionaux (Zone UEMOA, Pays de l'OHADA),
"Locale" et "NC", ainsi que les destinations combinées via transbordement
(Espagne/Royaume-Uni, France/Pays-Bas). 347 cellules modifiées, 77
libellés distincts au final (contre ~140 variantes). Documenté dans la
feuille Notes.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.####"/>
     <numFmt numFmtId="165" formatCode="#,##0.######"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,11 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -81,6 +86,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -797,6 +805,133 @@
       <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Le rapport ITIE 2018 indique par erreur l'unité "Tonne" pour la production ET l'exportation d'Or et d'Argent de PMC (156 925,68 "Tonnes" d'or et 10 114,22 "Tonnes" d'argent en production ; 143 389,00 et 9 323,50 en exportation), ce qui est physiquement impossible (156 925 tonnes d'or dépasseraient largement tout l'or jamais extrait dans le monde). Les quantités elles-mêmes sont cohérentes avec des onces troy (ordre de grandeur et valeur en FCFA/once compatibles avec le cours de l'or/argent de 2018 et avec la production de PMC les autres années). Ces 4 cellules ont donc été considérées comme des "Onces" mal étiquetées "Tonne" dans le rapport source, et l'unité a été corrigée en conséquence SANS multiplier la quantité (elle était déjà exprimée en onces).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Harmonisation des pays de destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Les rapports sources désignent parfois un même pays en anglais, en français, en majuscules ou avec des fautes de frappe selon l'année (ex : "China"/"CHINE"/"Chine", "Germany"/"ALLEMAGNE", "Ukranie"/"Ukraine"). Toutes ces variantes ont été unifiées sous un nom de pays canonique en français.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Cas particuliers</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Angleterre / England / United Kingdom / Royaume Uni</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Unifiés sous "Royaume-Uni".</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Hollande / Netherlands / Pays Bas</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Unifiés sous "Pays-Bas".</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Unifié sous "Suisse".</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Dubai / Dubaï / Emirats Arabes Unis</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Unifiés sous "Émirats Arabes Unis" (Dubai est utilisé comme raccourci du pays dans les rapports source).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>PARADIP INDIA / Lebanon - Beirut</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Simplifiés en "Inde" / "Liban" (le port ou la ville de destination indiqué par la source a été ramené au pays).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Zone UEMOA / Zone hors UEMOA, Pays de l'OHADA / Pays hors l'OHADA, Locale, NC</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Conservés tels quels : ce ne sont pas des pays mais des zones économiques régionales, des ventes locales ou une donnée non communiquée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Espagne/Angleterre, Espagne/France, Espagne/Hollande, France / Pays bas</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Destinations combinées (transbordement via un pays intermédiaire) conservées telles quelles dans le rapport source 2014-2016 ; seule l'orthographe des pays et le séparateur ("/") ont été harmonisés (ex : "Espagne/Royaume-Uni").</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Greenwich</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Conservé tel quel (destination ambiguë du rapport 2016, non réinterprétée faute de certitude).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Après harmonisation : 77 libellés de destination distincts sur la feuille exportation (contre environ 140 variantes avant harmonisation).</t>
         </is>
       </c>
     </row>
@@ -11593,7 +11728,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Benin</t>
+          <t>Bénin</t>
         </is>
       </c>
     </row>
@@ -11686,7 +11821,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Guinee Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -11717,7 +11852,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Guinée Conakry</t>
+          <t>Guinée</t>
         </is>
       </c>
     </row>
@@ -11903,7 +12038,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -11934,7 +12069,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>hors uemoa</t>
+          <t>Zone hors UEMOA</t>
         </is>
       </c>
     </row>
@@ -11965,7 +12100,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -11996,7 +12131,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -12120,7 +12255,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12286,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>RUSSIE</t>
+          <t>Russie</t>
         </is>
       </c>
     </row>
@@ -12182,7 +12317,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -12275,7 +12410,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -12554,7 +12689,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -12678,7 +12813,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -12709,7 +12844,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -12740,7 +12875,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -12802,7 +12937,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Espagne/Angleterre</t>
+          <t>Espagne/Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -12864,7 +12999,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Espagne/Hollande</t>
+          <t>Espagne/Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -12926,7 +13061,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -12988,7 +13123,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -13081,7 +13216,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Liberia</t>
+          <t>Libéria</t>
         </is>
       </c>
     </row>
@@ -13143,7 +13278,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>PARADIP INDIA</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -13515,7 +13650,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Sierra Léone</t>
+          <t>Sierra Leone</t>
         </is>
       </c>
     </row>
@@ -14104,7 +14239,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -14135,7 +14270,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>hors uemoa</t>
+          <t>Zone hors UEMOA</t>
         </is>
       </c>
     </row>
@@ -14259,7 +14394,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Sud Afrique</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -14321,7 +14456,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -14631,7 +14766,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -14662,7 +14797,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Sud Afrique</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -14755,7 +14890,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -15003,7 +15138,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -15127,7 +15262,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -15220,7 +15355,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -15344,7 +15479,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -15468,7 +15603,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -15499,7 +15634,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -15685,7 +15820,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -16491,7 +16626,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -16522,7 +16657,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>hors uemoa</t>
+          <t>Zone hors UEMOA</t>
         </is>
       </c>
     </row>
@@ -16677,7 +16812,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -16987,7 +17122,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -17113,7 +17248,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -17361,7 +17496,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -17423,7 +17558,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Afrique du sud</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17651,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -17578,7 +17713,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Thaïlande</t>
         </is>
       </c>
     </row>
@@ -17671,7 +17806,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -17826,7 +17961,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -17857,7 +17992,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Royaume Uni</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -18012,7 +18147,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>France / Pays bas</t>
+          <t>France/Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -18043,7 +18178,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -18074,7 +18209,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Royaume Uni</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -18198,7 +18333,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -18818,7 +18953,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -18849,7 +18984,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>hors uemoa</t>
+          <t>Zone hors UEMOA</t>
         </is>
       </c>
     </row>
@@ -18911,7 +19046,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Ukranie</t>
+          <t>Ukraine</t>
         </is>
       </c>
     </row>
@@ -18942,7 +19077,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Etats Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -19097,7 +19232,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -19128,7 +19263,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -19376,7 +19511,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -19469,7 +19604,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>Etats Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -19562,7 +19697,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -19748,7 +19883,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -19810,7 +19945,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Afrique de Sud</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -19872,7 +20007,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Etats Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -19965,7 +20100,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>Ukranie</t>
+          <t>Ukraine</t>
         </is>
       </c>
     </row>
@@ -19996,7 +20131,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>Etats Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -20058,7 +20193,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -20089,7 +20224,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -20337,7 +20472,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -20368,7 +20503,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>SOUTH KOREA</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -20399,7 +20534,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>SPAIN</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -20430,7 +20565,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>TURKEY</t>
+          <t>Turquie</t>
         </is>
       </c>
     </row>
@@ -20492,7 +20627,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Pays Bas</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -20523,7 +20658,7 @@
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>Royaume Uni</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -20647,7 +20782,7 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -20802,7 +20937,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>Etats Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -21360,7 +21495,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>UEMOA</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -21391,7 +21526,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>hors UEMOA</t>
+          <t>Zone hors UEMOA</t>
         </is>
       </c>
     </row>
@@ -21422,7 +21557,7 @@
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>AFRIQUE DU SUD</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -21453,7 +21588,7 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>ALLEMAGNE</t>
+          <t>Allemagne</t>
         </is>
       </c>
     </row>
@@ -21484,7 +21619,7 @@
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>ARABIE SAOUDITE</t>
+          <t>Arabie Saoudite</t>
         </is>
       </c>
     </row>
@@ -21515,7 +21650,7 @@
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>AUSTRALIE</t>
+          <t>Australie</t>
         </is>
       </c>
     </row>
@@ -21546,7 +21681,7 @@
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>BELGIQUE</t>
+          <t>Belgique</t>
         </is>
       </c>
     </row>
@@ -21577,7 +21712,7 @@
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>BRÉSIL</t>
+          <t>Brésil</t>
         </is>
       </c>
     </row>
@@ -21608,7 +21743,7 @@
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>CHINE</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -21639,7 +21774,7 @@
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>ESPAGNE</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -21670,7 +21805,7 @@
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>ÉTATS-UNIS</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -21701,7 +21836,7 @@
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -21732,7 +21867,7 @@
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -21763,7 +21898,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>INDONÉSIE</t>
+          <t>Indonésie</t>
         </is>
       </c>
     </row>
@@ -21794,7 +21929,7 @@
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>ITALIE</t>
+          <t>Italie</t>
         </is>
       </c>
     </row>
@@ -21825,7 +21960,7 @@
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>JAPON</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -21856,7 +21991,7 @@
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>MALAISIE</t>
+          <t>Malaisie</t>
         </is>
       </c>
     </row>
@@ -21887,7 +22022,7 @@
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>MEXIQUE</t>
+          <t>Mexique</t>
         </is>
       </c>
     </row>
@@ -21918,7 +22053,7 @@
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>MONTÉNÉGRO</t>
+          <t>Monténégro</t>
         </is>
       </c>
     </row>
@@ -21949,7 +22084,7 @@
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>NIGER</t>
+          <t>Niger</t>
         </is>
       </c>
     </row>
@@ -21980,7 +22115,7 @@
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>PAYS-BAS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -22011,7 +22146,7 @@
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>POLOGNE</t>
+          <t>Pologne</t>
         </is>
       </c>
     </row>
@@ -22042,7 +22177,7 @@
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>ROYAUME-UNI</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -22073,7 +22208,7 @@
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>SÉNÉGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -22104,7 +22239,7 @@
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>SUISSE</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -22135,7 +22270,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>UKRAINE</t>
+          <t>Ukraine</t>
         </is>
       </c>
     </row>
@@ -22197,7 +22332,7 @@
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>AFRIQUE DU SUD</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -22228,7 +22363,7 @@
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>ARABIE SAOUDITE</t>
+          <t>Arabie Saoudite</t>
         </is>
       </c>
     </row>
@@ -22259,7 +22394,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>BELGIQUE</t>
+          <t>Belgique</t>
         </is>
       </c>
     </row>
@@ -22290,7 +22425,7 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>CHINE</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -22321,7 +22456,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>COLOMBIE</t>
+          <t>Colombie</t>
         </is>
       </c>
     </row>
@@ -22352,7 +22487,7 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>RÉPUBLIQUE DE CORÉE</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -22383,7 +22518,7 @@
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>COSTA RICA</t>
+          <t>Costa Rica</t>
         </is>
       </c>
     </row>
@@ -22414,7 +22549,7 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>ÉMIRATS ARABES UNIS</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -22445,7 +22580,7 @@
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>ESPAGNE</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -22476,7 +22611,7 @@
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>ÉTATS-UNIS</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -22507,7 +22642,7 @@
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -22538,7 +22673,7 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>ÎLES VIERGES DES ÉTATS-UNIS</t>
+          <t>Îles Vierges des États-Unis</t>
         </is>
       </c>
     </row>
@@ -22569,7 +22704,7 @@
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -22600,7 +22735,7 @@
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>JAPON</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -22631,7 +22766,7 @@
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>MALAISIE</t>
+          <t>Malaisie</t>
         </is>
       </c>
     </row>
@@ -22662,7 +22797,7 @@
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -22693,7 +22828,7 @@
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>MAROC</t>
+          <t>Maroc</t>
         </is>
       </c>
     </row>
@@ -22724,7 +22859,7 @@
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>MEXIQUE</t>
+          <t>Mexique</t>
         </is>
       </c>
     </row>
@@ -22755,7 +22890,7 @@
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>MONTÉNÉGRO</t>
+          <t>Monténégro</t>
         </is>
       </c>
     </row>
@@ -22786,7 +22921,7 @@
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>NAURU</t>
+          <t>Nauru</t>
         </is>
       </c>
     </row>
@@ -22817,7 +22952,7 @@
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>NIGER</t>
+          <t>Niger</t>
         </is>
       </c>
     </row>
@@ -22848,7 +22983,7 @@
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>NORVÈGE</t>
+          <t>Norvège</t>
         </is>
       </c>
     </row>
@@ -22879,7 +23014,7 @@
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>PAYS-BAS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -22910,7 +23045,7 @@
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>POLOGNE</t>
+          <t>Pologne</t>
         </is>
       </c>
     </row>
@@ -22941,7 +23076,7 @@
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>SÉNÉGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -22972,7 +23107,7 @@
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>SUÈDE</t>
+          <t>Suède</t>
         </is>
       </c>
     </row>
@@ -23003,7 +23138,7 @@
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>SUISSE</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -23034,7 +23169,7 @@
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>UKRAINE</t>
+          <t>Ukraine</t>
         </is>
       </c>
     </row>
@@ -23127,7 +23262,7 @@
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>CHINE</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -23158,7 +23293,7 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>ÉMIRATS ARABES UNIS</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -23189,7 +23324,7 @@
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -23220,7 +23355,7 @@
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>CÔTE D'IVOIRE</t>
+          <t>Côte d'Ivoire</t>
         </is>
       </c>
     </row>
@@ -23251,7 +23386,7 @@
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>ÉTATS-UNIS</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -23282,7 +23417,7 @@
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>GUINÉE-BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -23313,7 +23448,7 @@
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>ITALIE</t>
+          <t>Italie</t>
         </is>
       </c>
     </row>
@@ -23344,7 +23479,7 @@
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -23375,7 +23510,7 @@
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t>SINGAPOUR</t>
+          <t>Singapour</t>
         </is>
       </c>
     </row>
@@ -23406,7 +23541,7 @@
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -23437,7 +23572,7 @@
       </c>
       <c r="G384" t="inlineStr">
         <is>
-          <t>GAMBIE</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -23468,7 +23603,7 @@
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>GUINEE BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -23499,7 +23634,7 @@
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -23530,7 +23665,7 @@
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>CAP-VERT</t>
+          <t>Cap-Vert</t>
         </is>
       </c>
     </row>
@@ -23561,7 +23696,7 @@
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>ROYAUME-UNI</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -23592,7 +23727,7 @@
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>LIBAN</t>
+          <t>Liban</t>
         </is>
       </c>
     </row>
@@ -23623,7 +23758,7 @@
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t>SWITZERLAND</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -23654,7 +23789,7 @@
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t>SWAZILAND</t>
+          <t>Swaziland</t>
         </is>
       </c>
     </row>
@@ -23685,7 +23820,7 @@
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t>ESPAGNE</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -23716,7 +23851,7 @@
       </c>
       <c r="G393" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -23747,7 +23882,7 @@
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t>ITALIE</t>
+          <t>Italie</t>
         </is>
       </c>
     </row>
@@ -23778,7 +23913,7 @@
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t>MALAISIE</t>
+          <t>Malaisie</t>
         </is>
       </c>
     </row>
@@ -23809,7 +23944,7 @@
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -23840,7 +23975,7 @@
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t>NOUVELLE-ZÉLANDE</t>
+          <t>Nouvelle-Zélande</t>
         </is>
       </c>
     </row>
@@ -23871,7 +24006,7 @@
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t>POLOGNE</t>
+          <t>Pologne</t>
         </is>
       </c>
     </row>
@@ -23902,7 +24037,7 @@
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t>SINGAPOUR</t>
+          <t>Singapour</t>
         </is>
       </c>
     </row>
@@ -24181,7 +24316,7 @@
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -24336,7 +24471,7 @@
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -24522,7 +24657,7 @@
       </c>
       <c r="G419" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -25173,7 +25308,7 @@
       </c>
       <c r="G440" t="inlineStr">
         <is>
-          <t>La Corée</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -25235,7 +25370,7 @@
       </c>
       <c r="G442" t="inlineStr">
         <is>
-          <t>Emirats Arabes Unis</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -25297,7 +25432,7 @@
       </c>
       <c r="G444" t="inlineStr">
         <is>
-          <t>Etats-Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -26010,7 +26145,7 @@
       </c>
       <c r="G467" t="inlineStr">
         <is>
-          <t>La Corée</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -26103,7 +26238,7 @@
       </c>
       <c r="G470" t="inlineStr">
         <is>
-          <t>Etats-Unis</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -27033,7 +27168,7 @@
       </c>
       <c r="G500" t="inlineStr">
         <is>
-          <t>Guinée Bissau</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -27192,7 +27327,7 @@
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -27254,7 +27389,7 @@
       </c>
       <c r="G507" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -27287,7 +27422,7 @@
       </c>
       <c r="G508" t="inlineStr">
         <is>
-          <t>Lebanon - Beirut</t>
+          <t>Liban</t>
         </is>
       </c>
     </row>
@@ -27320,7 +27455,7 @@
       </c>
       <c r="G509" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -27506,7 +27641,7 @@
       </c>
       <c r="G515" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Thaïlande</t>
         </is>
       </c>
     </row>
@@ -27537,7 +27672,7 @@
       </c>
       <c r="G516" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Australie</t>
         </is>
       </c>
     </row>
@@ -27568,7 +27703,7 @@
       </c>
       <c r="G517" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Brésil</t>
         </is>
       </c>
     </row>
@@ -27599,7 +27734,7 @@
       </c>
       <c r="G518" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -27630,7 +27765,7 @@
       </c>
       <c r="G519" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -27661,7 +27796,7 @@
       </c>
       <c r="G520" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -27723,7 +27858,7 @@
       </c>
       <c r="G522" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Allemagne</t>
         </is>
       </c>
     </row>
@@ -27754,7 +27889,7 @@
       </c>
       <c r="G523" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -27785,7 +27920,7 @@
       </c>
       <c r="G524" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Italie</t>
         </is>
       </c>
     </row>
@@ -27816,7 +27951,7 @@
       </c>
       <c r="G525" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -27847,7 +27982,7 @@
       </c>
       <c r="G526" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Malaisie</t>
         </is>
       </c>
     </row>
@@ -27878,7 +28013,7 @@
       </c>
       <c r="G527" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Mexique</t>
         </is>
       </c>
     </row>
@@ -27909,7 +28044,7 @@
       </c>
       <c r="G528" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -27940,7 +28075,7 @@
       </c>
       <c r="G529" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Norvège</t>
         </is>
       </c>
     </row>
@@ -27971,7 +28106,7 @@
       </c>
       <c r="G530" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -28002,7 +28137,7 @@
       </c>
       <c r="G531" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -28033,7 +28168,7 @@
       </c>
       <c r="G532" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -28064,7 +28199,7 @@
       </c>
       <c r="G533" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Turquie</t>
         </is>
       </c>
     </row>
@@ -28095,7 +28230,7 @@
       </c>
       <c r="G534" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -28467,7 +28602,7 @@
       </c>
       <c r="G546" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -28498,7 +28633,7 @@
       </c>
       <c r="G547" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -28529,7 +28664,7 @@
       </c>
       <c r="G548" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -28560,7 +28695,7 @@
       </c>
       <c r="G549" t="inlineStr">
         <is>
-          <t>NORWAY</t>
+          <t>Norvège</t>
         </is>
       </c>
     </row>
@@ -29056,7 +29191,7 @@
       </c>
       <c r="G565" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -29087,7 +29222,7 @@
       </c>
       <c r="G566" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -29118,7 +29253,7 @@
       </c>
       <c r="G567" t="inlineStr">
         <is>
-          <t>SPAIN</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -29149,7 +29284,7 @@
       </c>
       <c r="G568" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -29180,7 +29315,7 @@
       </c>
       <c r="G569" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -29242,7 +29377,7 @@
       </c>
       <c r="G571" t="inlineStr">
         <is>
-          <t>ITALY</t>
+          <t>Italie</t>
         </is>
       </c>
     </row>
@@ -29273,7 +29408,7 @@
       </c>
       <c r="G572" t="inlineStr">
         <is>
-          <t>TURKEY</t>
+          <t>Turquie</t>
         </is>
       </c>
     </row>
@@ -29304,7 +29439,7 @@
       </c>
       <c r="G573" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -29335,7 +29470,7 @@
       </c>
       <c r="G574" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Brésil</t>
         </is>
       </c>
     </row>
@@ -29366,7 +29501,7 @@
       </c>
       <c r="G575" t="inlineStr">
         <is>
-          <t>NETHERLANDS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -29397,7 +29532,7 @@
       </c>
       <c r="G576" t="inlineStr">
         <is>
-          <t>GERMANY</t>
+          <t>Allemagne</t>
         </is>
       </c>
     </row>
@@ -29428,7 +29563,7 @@
       </c>
       <c r="G577" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -29459,7 +29594,7 @@
       </c>
       <c r="G578" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -29490,7 +29625,7 @@
       </c>
       <c r="G579" t="inlineStr">
         <is>
-          <t>SPAIN</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -29521,7 +29656,7 @@
       </c>
       <c r="G580" t="inlineStr">
         <is>
-          <t>GERMANY</t>
+          <t>Allemagne</t>
         </is>
       </c>
     </row>
@@ -29552,7 +29687,7 @@
       </c>
       <c r="G581" t="inlineStr">
         <is>
-          <t>NETHERLANDS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -29583,7 +29718,7 @@
       </c>
       <c r="G582" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -29614,7 +29749,7 @@
       </c>
       <c r="G583" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -29645,7 +29780,7 @@
       </c>
       <c r="G584" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -29676,7 +29811,7 @@
       </c>
       <c r="G585" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -29707,7 +29842,7 @@
       </c>
       <c r="G586" t="inlineStr">
         <is>
-          <t>NORWAY</t>
+          <t>Norvège</t>
         </is>
       </c>
     </row>
@@ -29738,7 +29873,7 @@
       </c>
       <c r="G587" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -29769,7 +29904,7 @@
       </c>
       <c r="G588" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -29800,7 +29935,7 @@
       </c>
       <c r="G589" t="inlineStr">
         <is>
-          <t>SOUTH KOREA</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -29893,7 +30028,7 @@
       </c>
       <c r="G592" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -29955,7 +30090,7 @@
       </c>
       <c r="G594" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -29986,7 +30121,7 @@
       </c>
       <c r="G595" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -30017,7 +30152,7 @@
       </c>
       <c r="G596" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -30048,7 +30183,7 @@
       </c>
       <c r="G597" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -30079,7 +30214,7 @@
       </c>
       <c r="G598" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -30110,7 +30245,7 @@
       </c>
       <c r="G599" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -30141,7 +30276,7 @@
       </c>
       <c r="G600" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -30172,7 +30307,7 @@
       </c>
       <c r="G601" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -30203,7 +30338,7 @@
       </c>
       <c r="G602" t="inlineStr">
         <is>
-          <t>SOUTH KOREA</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -30234,7 +30369,7 @@
       </c>
       <c r="G603" t="inlineStr">
         <is>
-          <t>NETHERLANDS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -30265,7 +30400,7 @@
       </c>
       <c r="G604" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -30296,7 +30431,7 @@
       </c>
       <c r="G605" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -30327,7 +30462,7 @@
       </c>
       <c r="G606" t="inlineStr">
         <is>
-          <t>SOUTH AFRICA</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -30358,7 +30493,7 @@
       </c>
       <c r="G607" t="inlineStr">
         <is>
-          <t>GERMANY</t>
+          <t>Allemagne</t>
         </is>
       </c>
     </row>
@@ -30389,7 +30524,7 @@
       </c>
       <c r="G608" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -30420,7 +30555,7 @@
       </c>
       <c r="G609" t="inlineStr">
         <is>
-          <t>SOUTH KOREA</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
     </row>
@@ -30451,7 +30586,7 @@
       </c>
       <c r="G610" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>Japon</t>
         </is>
       </c>
     </row>
@@ -30482,7 +30617,7 @@
       </c>
       <c r="G611" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -30513,7 +30648,7 @@
       </c>
       <c r="G612" t="inlineStr">
         <is>
-          <t>NETHERLANDS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -30544,7 +30679,7 @@
       </c>
       <c r="G613" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Chine</t>
         </is>
       </c>
     </row>
@@ -30575,7 +30710,7 @@
       </c>
       <c r="G614" t="inlineStr">
         <is>
-          <t>TAIWAN</t>
+          <t>Taiwan</t>
         </is>
       </c>
     </row>
@@ -30606,7 +30741,7 @@
       </c>
       <c r="G615" t="inlineStr">
         <is>
-          <t>SPAIN</t>
+          <t>Espagne</t>
         </is>
       </c>
     </row>
@@ -30637,7 +30772,7 @@
       </c>
       <c r="G616" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -30668,7 +30803,7 @@
       </c>
       <c r="G617" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -30699,7 +30834,7 @@
       </c>
       <c r="G618" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -30730,7 +30865,7 @@
       </c>
       <c r="G619" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -30761,7 +30896,7 @@
       </c>
       <c r="G620" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -30792,7 +30927,7 @@
       </c>
       <c r="G621" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -30823,7 +30958,7 @@
       </c>
       <c r="G622" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -31261,7 +31396,7 @@
       </c>
       <c r="G636" t="inlineStr">
         <is>
-          <t>SUISSE</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -31292,7 +31427,7 @@
       </c>
       <c r="G637" t="inlineStr">
         <is>
-          <t>AUSTRALIE</t>
+          <t>Australie</t>
         </is>
       </c>
     </row>
@@ -31323,7 +31458,7 @@
       </c>
       <c r="G638" t="inlineStr">
         <is>
-          <t>SENEGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -31354,7 +31489,7 @@
       </c>
       <c r="G639" t="inlineStr">
         <is>
-          <t>INDIA</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -31385,7 +31520,7 @@
       </c>
       <c r="G640" t="inlineStr">
         <is>
-          <t>UNITED ARAB EMIRATES</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -31416,7 +31551,7 @@
       </c>
       <c r="G641" t="inlineStr">
         <is>
-          <t>SWITZERLAND</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -31447,7 +31582,7 @@
       </c>
       <c r="G642" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -31478,7 +31613,7 @@
       </c>
       <c r="G643" t="inlineStr">
         <is>
-          <t>GAMBIE</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -31509,7 +31644,7 @@
       </c>
       <c r="G644" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -31540,7 +31675,7 @@
       </c>
       <c r="G645" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -31571,7 +31706,7 @@
       </c>
       <c r="G646" t="inlineStr">
         <is>
-          <t>GAMBIE</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -31602,7 +31737,7 @@
       </c>
       <c r="G647" t="inlineStr">
         <is>
-          <t>GAMBIE</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -31633,7 +31768,7 @@
       </c>
       <c r="G648" t="inlineStr">
         <is>
-          <t>MAURITANIE</t>
+          <t>Mauritanie</t>
         </is>
       </c>
     </row>
@@ -31664,7 +31799,7 @@
       </c>
       <c r="G649" t="inlineStr">
         <is>
-          <t>GUINEE BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -31695,7 +31830,7 @@
       </c>
       <c r="G650" t="inlineStr">
         <is>
-          <t>MAURITANIE</t>
+          <t>Mauritanie</t>
         </is>
       </c>
     </row>
@@ -31726,7 +31861,7 @@
       </c>
       <c r="G651" t="inlineStr">
         <is>
-          <t>GUINEE BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -31757,7 +31892,7 @@
       </c>
       <c r="G652" t="inlineStr">
         <is>
-          <t>GUINEE</t>
+          <t>Guinée</t>
         </is>
       </c>
     </row>
@@ -31788,7 +31923,7 @@
       </c>
       <c r="G653" t="inlineStr">
         <is>
-          <t>GUINEE-BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -31819,7 +31954,7 @@
       </c>
       <c r="G654" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -31850,7 +31985,7 @@
       </c>
       <c r="G655" t="inlineStr">
         <is>
-          <t>SWITZERLAND</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -31881,7 +32016,7 @@
       </c>
       <c r="G656" t="inlineStr">
         <is>
-          <t>SWITZERLAND</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -31912,7 +32047,7 @@
       </c>
       <c r="G657" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -31943,7 +32078,7 @@
       </c>
       <c r="G658" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -31974,7 +32109,7 @@
       </c>
       <c r="G659" t="inlineStr">
         <is>
-          <t>SENEGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -32005,7 +32140,7 @@
       </c>
       <c r="G660" t="inlineStr">
         <is>
-          <t>LITHUANIA</t>
+          <t>Lituanie</t>
         </is>
       </c>
     </row>
@@ -32036,7 +32171,7 @@
       </c>
       <c r="G661" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32067,7 +32202,7 @@
       </c>
       <c r="G662" t="inlineStr">
         <is>
-          <t>SENEGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -32098,7 +32233,7 @@
       </c>
       <c r="G663" t="inlineStr">
         <is>
-          <t>GHANA</t>
+          <t>Ghana</t>
         </is>
       </c>
     </row>
@@ -32129,7 +32264,7 @@
       </c>
       <c r="G664" t="inlineStr">
         <is>
-          <t>EL SALVADOR</t>
+          <t>El Salvador</t>
         </is>
       </c>
     </row>
@@ -32160,7 +32295,7 @@
       </c>
       <c r="G665" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32191,7 +32326,7 @@
       </c>
       <c r="G666" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32222,7 +32357,7 @@
       </c>
       <c r="G667" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32253,7 +32388,7 @@
       </c>
       <c r="G668" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32284,7 +32419,7 @@
       </c>
       <c r="G669" t="inlineStr">
         <is>
-          <t>GAMBIA</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -32315,7 +32450,7 @@
       </c>
       <c r="G670" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32481,7 @@
       </c>
       <c r="G671" t="inlineStr">
         <is>
-          <t>ANGLETERRE</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -32377,7 +32512,7 @@
       </c>
       <c r="G672" t="inlineStr">
         <is>
-          <t>PAYS-BAS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -32408,7 +32543,7 @@
       </c>
       <c r="G673" t="inlineStr">
         <is>
-          <t>SENEGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32574,7 @@
       </c>
       <c r="G674" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32470,7 +32605,7 @@
       </c>
       <c r="G675" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32501,7 +32636,7 @@
       </c>
       <c r="G676" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32565,7 +32700,7 @@
       </c>
       <c r="G678" t="inlineStr">
         <is>
-          <t>SENEGAL</t>
+          <t>Sénégal</t>
         </is>
       </c>
     </row>
@@ -32596,7 +32731,7 @@
       </c>
       <c r="G679" t="inlineStr">
         <is>
-          <t>GAMBIE</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -32629,7 +32764,7 @@
       </c>
       <c r="G680" t="inlineStr">
         <is>
-          <t>GAMBIE</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -32660,7 +32795,7 @@
       </c>
       <c r="G681" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -32691,7 +32826,7 @@
       </c>
       <c r="G682" t="inlineStr">
         <is>
-          <t>SUISSE</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -32722,7 +32857,7 @@
       </c>
       <c r="G683" t="inlineStr">
         <is>
-          <t>AUSTRALIE</t>
+          <t>Australie</t>
         </is>
       </c>
     </row>
@@ -32753,7 +32888,7 @@
       </c>
       <c r="G684" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32784,7 +32919,7 @@
       </c>
       <c r="G685" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32815,7 +32950,7 @@
       </c>
       <c r="G686" t="inlineStr">
         <is>
-          <t>MALI</t>
+          <t>Mali</t>
         </is>
       </c>
     </row>
@@ -32846,7 +32981,7 @@
       </c>
       <c r="G687" t="inlineStr">
         <is>
-          <t>GUINEA-BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -32877,7 +33012,7 @@
       </c>
       <c r="G688" t="inlineStr">
         <is>
-          <t>BURKINA FASO</t>
+          <t>Burkina Faso</t>
         </is>
       </c>
     </row>
@@ -32908,7 +33043,7 @@
       </c>
       <c r="G689" t="inlineStr">
         <is>
-          <t>INDIA</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -32970,7 +33105,7 @@
       </c>
       <c r="G691" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -33032,7 +33167,7 @@
       </c>
       <c r="G693" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -33063,7 +33198,7 @@
       </c>
       <c r="G694" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -33094,7 +33229,7 @@
       </c>
       <c r="G695" t="inlineStr">
         <is>
-          <t>zone uemoa</t>
+          <t>Zone UEMOA</t>
         </is>
       </c>
     </row>
@@ -33125,7 +33260,7 @@
       </c>
       <c r="G696" t="inlineStr">
         <is>
-          <t>zone hors uemoa</t>
+          <t>Zone hors UEMOA</t>
         </is>
       </c>
     </row>
@@ -33218,7 +33353,7 @@
       </c>
       <c r="G699" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -33249,7 +33384,7 @@
       </c>
       <c r="G700" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -33311,7 +33446,7 @@
       </c>
       <c r="G702" t="inlineStr">
         <is>
-          <t>GUINEE BISSAU</t>
+          <t>Guinée-Bissau</t>
         </is>
       </c>
     </row>
@@ -33404,7 +33539,7 @@
       </c>
       <c r="G705" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -33435,7 +33570,7 @@
       </c>
       <c r="G706" t="inlineStr">
         <is>
-          <t>INDE</t>
+          <t>Inde</t>
         </is>
       </c>
     </row>
@@ -33466,7 +33601,7 @@
       </c>
       <c r="G707" t="inlineStr">
         <is>
-          <t>SWITZERLAND</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -33497,7 +33632,7 @@
       </c>
       <c r="G708" t="inlineStr">
         <is>
-          <t>PAYS BAS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -33528,7 +33663,7 @@
       </c>
       <c r="G709" t="inlineStr">
         <is>
-          <t>INDONESIA</t>
+          <t>Indonésie</t>
         </is>
       </c>
     </row>
@@ -33559,7 +33694,7 @@
       </c>
       <c r="G710" t="inlineStr">
         <is>
-          <t>BRAZIL</t>
+          <t>Brésil</t>
         </is>
       </c>
     </row>
@@ -33621,7 +33756,7 @@
       </c>
       <c r="G712" t="inlineStr">
         <is>
-          <t>GHANA</t>
+          <t>Ghana</t>
         </is>
       </c>
     </row>
@@ -33714,7 +33849,7 @@
       </c>
       <c r="G715" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -33745,7 +33880,7 @@
       </c>
       <c r="G716" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Suisse</t>
         </is>
       </c>
     </row>
@@ -33776,7 +33911,7 @@
       </c>
       <c r="G717" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -33807,7 +33942,7 @@
       </c>
       <c r="G718" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -33900,7 +34035,7 @@
       </c>
       <c r="G721" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -33931,7 +34066,7 @@
       </c>
       <c r="G722" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -33962,7 +34097,7 @@
       </c>
       <c r="G723" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -33993,7 +34128,7 @@
       </c>
       <c r="G724" t="inlineStr">
         <is>
-          <t>PAYS BAS</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -34024,7 +34159,7 @@
       </c>
       <c r="G725" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -34057,7 +34192,7 @@
       </c>
       <c r="G726" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -34088,7 +34223,7 @@
       </c>
       <c r="G727" t="inlineStr">
         <is>
-          <t>Gambia</t>
+          <t>Gambie</t>
         </is>
       </c>
     </row>
@@ -34119,7 +34254,7 @@
       </c>
       <c r="G728" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34150,7 +34285,7 @@
       </c>
       <c r="G729" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34181,7 +34316,7 @@
       </c>
       <c r="G730" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34212,7 +34347,7 @@
       </c>
       <c r="G731" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34243,7 +34378,7 @@
       </c>
       <c r="G732" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34274,7 +34409,7 @@
       </c>
       <c r="G733" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34305,7 +34440,7 @@
       </c>
       <c r="G734" t="inlineStr">
         <is>
-          <t>FRANCE</t>
+          <t>France</t>
         </is>
       </c>
     </row>
@@ -34398,7 +34533,7 @@
       </c>
       <c r="G737" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -35266,7 +35401,7 @@
       </c>
       <c r="G765" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -35328,7 +35463,7 @@
       </c>
       <c r="G767" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -35359,7 +35494,7 @@
       </c>
       <c r="G768" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -35421,7 +35556,7 @@
       </c>
       <c r="G770" t="inlineStr">
         <is>
-          <t>Hollande</t>
+          <t>Pays-Bas</t>
         </is>
       </c>
     </row>
@@ -35799,7 +35934,7 @@
       </c>
       <c r="G782" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -35861,7 +35996,7 @@
       </c>
       <c r="G784" t="inlineStr">
         <is>
-          <t>Dubaï</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -35892,7 +36027,7 @@
       </c>
       <c r="G785" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -36047,7 +36182,7 @@
       </c>
       <c r="G790" t="inlineStr">
         <is>
-          <t>Afrique de Sud</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -36423,7 +36558,7 @@
       </c>
       <c r="G802" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -36609,7 +36744,7 @@
       </c>
       <c r="G808" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>
@@ -36857,7 +36992,7 @@
       </c>
       <c r="G816" t="inlineStr">
         <is>
-          <t>Afrique de Sud</t>
+          <t>Afrique du Sud</t>
         </is>
       </c>
     </row>
@@ -36950,7 +37085,7 @@
       </c>
       <c r="G819" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>États-Unis</t>
         </is>
       </c>
     </row>
@@ -37012,7 +37147,7 @@
       </c>
       <c r="G821" t="inlineStr">
         <is>
-          <t>Dubaï</t>
+          <t>Émirats Arabes Unis</t>
         </is>
       </c>
     </row>
@@ -37043,7 +37178,7 @@
       </c>
       <c r="G822" t="inlineStr">
         <is>
-          <t>Angleterre</t>
+          <t>Royaume-Uni</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Convertit aussi l'Or/l'Argent en Tonne pour une unité unique
Poursuit l'harmonisation des unités : les 77 lignes encore en Once
(once troy) pour l'Or et l'Argent sont converties en Tonne, comme le
reste des feuilles (1 Tonne = 32 150,7466 onces troy, via 1 once =
31,1034768 g). Une seule unité de poids (Tonne) subsiste désormais sur
les deux feuilles, avec Mètre cube conservé à part pour les volumes.
Met à jour la feuille Notes en conséquence.
</commit_message>
<xml_diff>
--- a/Données sur la production et les ventes.xlsx
+++ b/Données sur la production et les ventes.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.####"/>
     <numFmt numFmtId="165" formatCode="#,##0.######"/>
+    <numFmt numFmtId="166" formatCode="#,##0.########"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -68,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -89,6 +90,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -510,6 +512,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -524,6 +527,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -591,6 +595,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -646,6 +651,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
@@ -739,6 +745,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
@@ -746,6 +753,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
@@ -780,7 +788,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Unité cible : Once (once troy). Conversion utilisée : 1 once troy = 31,1034768 grammes (valeur standard internationale). Kg converti en once via les grammes (Kg × 1 000 / 31,1034768) ; Gramme converti directement (Gramme / 31,1034768) ; Tonne convertie en once (Tonne × 1 000 000 / 31,1034768, soit environ × 32 150,7466).</t>
+          <t>Convertis en Tonne, comme le reste de la feuille (une seule unité de poids sur tout le classeur). Conversion utilisée : 1 once troy = 31,1034768 grammes (valeur standard internationale), donc 1 Tonne = 1 000 000 g / 31,1034768 = 32 150,7466 onces troy. Les quantités initialement en Once/Onces/Ounce/Onces troy (Oz), Kg ou Gramme ont toutes été ramenées en Tonne via les grammes.</t>
         </is>
       </c>
     </row>
@@ -925,13 +933,17 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-    </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>Après harmonisation : 77 libellés de destination distincts sur la feuille exportation (contre environ 140 variantes avant harmonisation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Mise à jour : les quantités d'Or/Argent, initialement conservées en Once (once troy) lors d'une première passe d'harmonisation, ont finalement aussi été converties en Tonne pour qu'une seule unité de poids (Tonne) soit utilisée sur l'ensemble des deux feuilles (avec Mètre cube conservé à part pour les volumes).</t>
         </is>
       </c>
     </row>
@@ -1107,11 +1119,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>211823</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>6.58843177</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>132680295481</v>
@@ -1138,7 +1150,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Once</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1964,11 +1976,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>182282</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="n">
+        <v>5.66960396</v>
       </c>
       <c r="F32" s="4" t="n">
         <v>125343600170</v>
@@ -1995,7 +2007,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Once</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2823,11 +2835,11 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="n">
-        <v>216735</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="n">
+        <v>6.74121204</v>
       </c>
       <c r="F59" s="4" t="n">
         <v>158275855422</v>
@@ -2854,7 +2866,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Once</t>
+          <t>Tonne</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3752,11 +3764,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="n">
-        <v>233119</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E88" s="10" t="n">
+        <v>7.25081141</v>
       </c>
       <c r="F88" s="4" t="n">
         <v>170115735962</v>
@@ -3783,11 +3795,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E89" s="4" t="n">
-        <v>21222</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="n">
+        <v>0.66007798</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>207254807</v>
@@ -4665,11 +4677,11 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="n">
-        <v>245304.5</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E117" s="10" t="n">
+        <v>7.62982282</v>
       </c>
       <c r="F117" s="4" t="n">
         <v>169627487970</v>
@@ -4696,11 +4708,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E118" s="5" t="n">
-        <v>20254.5</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="n">
+        <v>0.62998537</v>
       </c>
       <c r="F118" s="4" t="n">
         <v>175186261</v>
@@ -5435,11 +5447,11 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E141" s="5" t="n">
-        <v>156925.68</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E141" s="10" t="n">
+        <v>4.88093425</v>
       </c>
       <c r="F141" s="4" t="n">
         <v>100910301956</v>
@@ -5466,11 +5478,11 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E142" s="5" t="n">
-        <v>10114.22</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E142" s="10" t="n">
+        <v>0.31458741</v>
       </c>
       <c r="F142" s="4" t="n">
         <v>79470206</v>
@@ -6117,11 +6129,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E163" s="4" t="n">
-        <v>12527</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="n">
+        <v>0.38963325</v>
       </c>
       <c r="F163" s="4" t="n">
         <v>119665719</v>
@@ -6148,11 +6160,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E164" s="4" t="n">
-        <v>180980</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="n">
+        <v>5.62910723</v>
       </c>
       <c r="F164" s="4" t="n">
         <v>147874140109</v>
@@ -6210,11 +6222,11 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E166" s="4" t="n">
-        <v>17557</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="n">
+        <v>0.54608374</v>
       </c>
       <c r="F166" s="4" t="n">
         <v>165428598</v>
@@ -6241,11 +6253,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E167" s="4" t="n">
-        <v>234355</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="n">
+        <v>7.28925531</v>
       </c>
       <c r="F167" s="4" t="n">
         <v>189854215168</v>
@@ -6427,11 +6439,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E173" s="5" t="n">
-        <v>225055.226</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="F173" s="4" t="n">
         <v>217680000000</v>
@@ -6458,11 +6470,11 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E174" s="5" t="n">
-        <v>186474.3301</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="n">
+        <v>5.8</v>
       </c>
       <c r="F174" s="4" t="n">
         <v>179340000000</v>
@@ -7210,11 +7222,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E198" s="5" t="n">
-        <v>392239.1081</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E198" s="10" t="n">
+        <v>12.2</v>
       </c>
       <c r="F198" s="4" t="n">
         <v>390697165834</v>
@@ -7241,11 +7253,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E199" s="5" t="n">
-        <v>32150.7466</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E199" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="F199" s="4" t="n">
         <v>453360287</v>
@@ -7272,11 +7284,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E200" s="5" t="n">
-        <v>128602.9863</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E200" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="F200" t="inlineStr">
         <is>
@@ -7305,11 +7317,11 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E201" s="5" t="n">
-        <v>9645.224</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E201" s="10" t="n">
+        <v>0.3</v>
       </c>
       <c r="F201" s="4" t="n">
         <v>130156827</v>
@@ -8146,11 +8158,11 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E228" s="5" t="n">
-        <v>353658.2123</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E228" s="10" t="n">
+        <v>11</v>
       </c>
       <c r="F228" s="4" t="n">
         <v>393709507828</v>
@@ -8177,11 +8189,11 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E229" s="5" t="n">
-        <v>129422.8303</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E229" s="10" t="n">
+        <v>4.0255</v>
       </c>
       <c r="F229" s="4" t="n">
         <v>145989168041</v>
@@ -8208,11 +8220,11 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E230" s="5" t="n">
-        <v>1559.3112</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E230" s="10" t="n">
+        <v>0.0485</v>
       </c>
       <c r="F230" t="inlineStr">
         <is>
@@ -9020,11 +9032,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E256" s="5" t="n">
-        <v>32150.7466</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E256" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="F256" s="4" t="n">
         <v>382666065</v>
@@ -9051,11 +9063,11 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E257" s="5" t="n">
-        <v>10461.8529</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E257" s="10" t="n">
+        <v>0.3254</v>
       </c>
       <c r="F257" s="4" t="n">
         <v>142020334</v>
@@ -9212,11 +9224,11 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E262" s="4" t="n">
-        <v>293680</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E262" s="10" t="n">
+        <v>9.13446907</v>
       </c>
       <c r="F262" s="4" t="n">
         <v>345263735282</v>
@@ -9243,11 +9255,11 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E263" s="4" t="n">
-        <v>22634</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E263" s="10" t="n">
+        <v>0.70399609</v>
       </c>
       <c r="F263" s="4" t="n">
         <v>316892931</v>
@@ -9468,11 +9480,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E270" s="4" t="n">
-        <v>119846</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E270" s="10" t="n">
+        <v>3.72762728</v>
       </c>
       <c r="F270" s="4" t="n">
         <v>139146872008</v>
@@ -9499,11 +9511,11 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E271" s="4" t="n">
-        <v>8951</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E271" s="10" t="n">
+        <v>0.27840722</v>
       </c>
       <c r="F271" s="4" t="n">
         <v>123303770</v>
@@ -10422,11 +10434,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E300" s="5" t="n">
-        <v>1796.6802</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E300" s="10" t="n">
+        <v>0.055883</v>
       </c>
       <c r="F300" t="inlineStr">
         <is>
@@ -10455,11 +10467,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E301" s="5" t="n">
-        <v>96.42010000000001</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E301" s="10" t="n">
+        <v>0.002999</v>
       </c>
       <c r="F301" t="inlineStr">
         <is>
@@ -10581,11 +10593,11 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E305" s="4" t="n">
-        <v>229115</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E305" s="10" t="n">
+        <v>7.12627309</v>
       </c>
       <c r="F305" s="4" t="n">
         <v>336554241516</v>
@@ -10612,11 +10624,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E306" s="4" t="n">
-        <v>18451</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E306" s="10" t="n">
+        <v>0.57389025</v>
       </c>
       <c r="F306" s="4" t="n">
         <v>311205277</v>
@@ -11139,11 +11151,11 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E323" s="4" t="n">
-        <v>123945</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E323" s="10" t="n">
+        <v>3.85512043</v>
       </c>
       <c r="F323" s="4" t="n">
         <v>83475795667</v>
@@ -11591,11 +11603,11 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E337" s="5" t="n">
-        <v>1656.9209</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E337" s="10" t="n">
+        <v>0.051536</v>
       </c>
       <c r="F337" t="inlineStr">
         <is>
@@ -11965,11 +11977,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>206336</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>6.41776699</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>129315030912</v>
@@ -11996,11 +12008,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>37209</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>1.15732927</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>355030358</v>
@@ -14166,11 +14178,11 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E81" s="4" t="n">
-        <v>193218</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E81" s="10" t="n">
+        <v>6.00975158</v>
       </c>
       <c r="F81" s="4" t="n">
         <v>132762285276</v>
@@ -14197,11 +14209,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E82" s="4" t="n">
-        <v>17887</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="n">
+        <v>0.55634789</v>
       </c>
       <c r="F82" s="4" t="n">
         <v>164774191</v>
@@ -16553,11 +16565,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E158" s="4" t="n">
-        <v>217652</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="n">
+        <v>6.76973393</v>
       </c>
       <c r="F158" s="4" t="n">
         <v>158823700311</v>
@@ -16584,11 +16596,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E159" s="4" t="n">
-        <v>18734</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="n">
+        <v>0.58269253</v>
       </c>
       <c r="F159" s="4" t="n">
         <v>199447095</v>
@@ -18880,11 +18892,11 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E233" s="4" t="n">
-        <v>231104</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E233" s="10" t="n">
+        <v>7.1881379</v>
       </c>
       <c r="F233" s="4" t="n">
         <v>168342880233</v>
@@ -18911,11 +18923,11 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E234" s="4" t="n">
-        <v>20448</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E234" s="10" t="n">
+        <v>0.63600389</v>
       </c>
       <c r="F234" s="4" t="n">
         <v>200690857</v>
@@ -21422,11 +21434,11 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E315" s="5" t="n">
-        <v>246306.69</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E315" s="10" t="n">
+        <v>7.66099442</v>
       </c>
       <c r="F315" s="4" t="n">
         <v>175925907803</v>
@@ -21453,11 +21465,11 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E316" s="5" t="n">
-        <v>20705.07</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E316" s="10" t="n">
+        <v>0.64399966</v>
       </c>
       <c r="F316" s="4" t="n">
         <v>182474962</v>
@@ -24088,11 +24100,11 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E401" s="5" t="n">
-        <v>143389</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E401" s="10" t="n">
+        <v>4.45989643</v>
       </c>
       <c r="F401" s="4" t="n">
         <v>101780154907</v>
@@ -24119,11 +24131,11 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E402" s="5" t="n">
-        <v>9323.5</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E402" s="10" t="n">
+        <v>0.28999327</v>
       </c>
       <c r="F402" s="4" t="n">
         <v>80632431</v>
@@ -24739,11 +24751,11 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E422" s="5" t="n">
-        <v>200009.7944</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E422" s="10" t="n">
+        <v>6.221</v>
       </c>
       <c r="F422" s="4" t="n">
         <v>151885748355</v>
@@ -24770,11 +24782,11 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E423" s="5" t="n">
-        <v>252222.6068</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E423" s="10" t="n">
+        <v>7.845</v>
       </c>
       <c r="F423" s="4" t="n">
         <v>189853050512</v>
@@ -26723,11 +26735,11 @@
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E486" s="4" t="n">
-        <v>128355</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E486" s="10" t="n">
+        <v>3.99228676</v>
       </c>
       <c r="F486" s="4" t="n">
         <v>117267141286</v>
@@ -26754,11 +26766,11 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E487" s="4" t="n">
-        <v>42455</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E487" s="10" t="n">
+        <v>1.32049811</v>
       </c>
       <c r="F487" s="4" t="n">
         <v>39522643736</v>
@@ -26785,11 +26797,11 @@
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E488" s="4" t="n">
-        <v>8500</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E488" s="10" t="n">
+        <v>0.26437955</v>
       </c>
       <c r="F488" s="4" t="n">
         <v>8692666730</v>
@@ -26816,11 +26828,11 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E489" s="4" t="n">
-        <v>217890</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E489" s="10" t="n">
+        <v>6.77713656</v>
       </c>
       <c r="F489" s="4" t="n">
         <v>220079268751</v>
@@ -26847,11 +26859,11 @@
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E490" s="4" t="n">
-        <v>18983</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E490" s="10" t="n">
+        <v>0.5904373000000001</v>
       </c>
       <c r="F490" s="4" t="n">
         <v>219911782</v>
@@ -26878,11 +26890,11 @@
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E491" s="4" t="n">
-        <v>16066</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E491" s="10" t="n">
+        <v>0.49970846</v>
       </c>
       <c r="F491" s="4" t="n">
         <v>193308323</v>
@@ -28529,11 +28541,11 @@
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E544" s="5" t="n">
-        <v>338920.31</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E544" s="10" t="n">
+        <v>10.5416</v>
       </c>
       <c r="F544" s="4" t="n">
         <v>380045730082</v>
@@ -28560,11 +28572,11 @@
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E545" s="5" t="n">
-        <v>129628.5951</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E545" s="10" t="n">
+        <v>4.0319</v>
       </c>
       <c r="F545" s="4" t="n">
         <v>147954684761</v>
@@ -28591,11 +28603,11 @@
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E546" s="5" t="n">
-        <v>11204.5352</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E546" s="10" t="n">
+        <v>0.3485</v>
       </c>
       <c r="F546" s="4" t="n">
         <v>12540974385</v>
@@ -31166,11 +31178,11 @@
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E629" s="4" t="n">
-        <v>27299</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E629" s="10" t="n">
+        <v>0.8490938099999999</v>
       </c>
       <c r="F629" s="4" t="n">
         <v>374908490</v>
@@ -31197,11 +31209,11 @@
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E630" s="4" t="n">
-        <v>11395</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E630" s="10" t="n">
+        <v>0.35442412</v>
       </c>
       <c r="F630" s="4" t="n">
         <v>143623609</v>
@@ -31385,11 +31397,11 @@
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E636" s="4" t="n">
-        <v>288697</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E636" s="10" t="n">
+        <v>8.97948044</v>
       </c>
       <c r="F636" s="4" t="n">
         <v>344273384269</v>
@@ -31416,11 +31428,11 @@
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E637" s="4" t="n">
-        <v>119950</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E637" s="10" t="n">
+        <v>3.73086204</v>
       </c>
       <c r="F637" s="4" t="n">
         <v>138107655558</v>
@@ -31447,11 +31459,11 @@
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E638" s="4" t="n">
-        <v>8000</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E638" s="10" t="n">
+        <v>0.24882781</v>
       </c>
       <c r="F638" s="4" t="n">
         <v>9494006760</v>
@@ -32815,11 +32827,11 @@
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E682" s="4" t="n">
-        <v>21822</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E682" s="10" t="n">
+        <v>0.67874007</v>
       </c>
       <c r="F682" s="4" t="n">
         <v>307938113</v>
@@ -32846,11 +32858,11 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E683" s="4" t="n">
-        <v>8872</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E683" s="10" t="n">
+        <v>0.27595005</v>
       </c>
       <c r="F683" s="4" t="n">
         <v>122375993</v>
@@ -33063,11 +33075,11 @@
       </c>
       <c r="D690" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E690" s="4" t="n">
-        <v>121623</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E690" s="10" t="n">
+        <v>3.78289816</v>
       </c>
       <c r="F690" s="4" t="n">
         <v>176892827875</v>
@@ -33094,11 +33106,11 @@
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E691" s="4" t="n">
-        <v>116418</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E691" s="10" t="n">
+        <v>3.62100456</v>
       </c>
       <c r="F691" s="4" t="n">
         <v>171988995312</v>
@@ -33125,11 +33137,11 @@
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E692" s="4" t="n">
-        <v>105001</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E692" s="10" t="n">
+        <v>3.26589617</v>
       </c>
       <c r="F692" s="4" t="n">
         <v>153070817850</v>
@@ -34491,11 +34503,11 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E736" s="4" t="n">
-        <v>10095</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E736" s="10" t="n">
+        <v>0.3139896</v>
       </c>
       <c r="F736" s="4" t="n">
         <v>169980320</v>
@@ -34522,11 +34534,11 @@
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E737" s="4" t="n">
-        <v>8904</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E737" s="10" t="n">
+        <v>0.27694536</v>
       </c>
       <c r="F737" s="4" t="n">
         <v>156146734</v>
@@ -34553,11 +34565,11 @@
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E738" s="4" t="n">
-        <v>8181</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E738" s="10" t="n">
+        <v>0.25445754</v>
       </c>
       <c r="F738" s="4" t="n">
         <v>140740539</v>
@@ -34615,11 +34627,11 @@
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E740" s="4" t="n">
-        <v>128393</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E740" s="10" t="n">
+        <v>3.9934687</v>
       </c>
       <c r="F740" s="4" t="n">
         <v>123373225492</v>
@@ -34646,11 +34658,11 @@
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E741" s="4" t="n">
-        <v>381943</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E741" s="10" t="n">
+        <v>11.87975524</v>
       </c>
       <c r="F741" s="4" t="n">
         <v>381693870501</v>
@@ -34677,11 +34689,11 @@
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E742" s="4" t="n">
-        <v>9257</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E742" s="10" t="n">
+        <v>0.28792488</v>
       </c>
       <c r="F742" s="4" t="n">
         <v>129692515</v>
@@ -34708,11 +34720,11 @@
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Once</t>
-        </is>
-      </c>
-      <c r="E743" s="4" t="n">
-        <v>33010</v>
+          <t>Tonne</t>
+        </is>
+      </c>
+      <c r="E743" s="10" t="n">
+        <v>1.02672577</v>
       </c>
       <c r="F743" s="4" t="n">
         <v>453060509</v>

</xml_diff>